<commit_message>
Agregar Cuadro de Vigas y Riostras por TIPOS (diseno por grupos de solicitacion, no una sola viga)
</commit_message>
<xml_diff>
--- a/Proyectos/Diseno-Estructural/Insumos/Diseno-Estructural-Calculos.xlsx
+++ b/Proyectos/Diseno-Estructural/Insumos/Diseno-Estructural-Calculos.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="Irregularidades" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Diseno Vigas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Diseno Riostras" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Diseno Viguetas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Cuadro Vigas-Riostras" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Diseno Vigas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Diseno Riostras" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Diseno Viguetas" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -61,6 +62,11 @@
       <name val="Aptos Narrow"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -95,7 +101,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -109,11 +115,74 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -158,6 +227,42 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -560,10 +665,34 @@
           <t>Sistema: PORTICOS RESISTENTES A MOMENTOS DE CONCRETO REFORZADO con capacidad MODERADA de disipacion de energia (DMO), en las dos direcciones, que resisten cargas gravitacionales y sismicas (NSR-10 Tabla A.3-3). Componentes: columnas (C1ESQ, C2BOR, C3INT, C4DIAG), vigas de carga VC 40x30, vigas de rigidez VR 40x35, entrepiso en losa aligerada en una direccion (vigueta h=0.34 + caseton + loseta 0.06 m). Materiales: f'c=28 MPa, fy=420 MPa. Localizacion: Santa Marta (amenaza sismica intermedia).</t>
         </is>
       </c>
-    </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
+      <c r="C5" s="16" t="n"/>
+      <c r="D5" s="16" t="n"/>
+      <c r="E5" s="16" t="n"/>
+      <c r="F5" s="16" t="n"/>
+      <c r="G5" s="16" t="n"/>
+      <c r="H5" s="16" t="n"/>
+      <c r="I5" s="16" t="n"/>
+      <c r="J5" s="17" t="n"/>
+    </row>
+    <row r="6">
+      <c r="B6" s="18" t="n"/>
+      <c r="J6" s="19" t="n"/>
+    </row>
+    <row r="7">
+      <c r="B7" s="18" t="n"/>
+      <c r="J7" s="19" t="n"/>
+    </row>
+    <row r="8">
+      <c r="B8" s="20" t="n"/>
+      <c r="C8" s="21" t="n"/>
+      <c r="D8" s="21" t="n"/>
+      <c r="E8" s="21" t="n"/>
+      <c r="F8" s="21" t="n"/>
+      <c r="G8" s="21" t="n"/>
+      <c r="H8" s="21" t="n"/>
+      <c r="I8" s="21" t="n"/>
+      <c r="J8" s="22" t="n"/>
+    </row>
     <row r="10">
       <c r="B10" s="4" t="inlineStr">
         <is>
@@ -1165,8 +1294,26 @@
           <t>CONCLUSION: estructura REGULAR en planta y altura. Torsion dmax/dprom = 1.02(X) y 1.01(Y) &lt; 1.20; masa 1.32 &lt; 1.50; rigidez creciente hacia la base; diafragma &lt; 50% area; retrocesos &lt; 15%. Por tanto phi_p = phi_a = phi_r = 1.0 y R = 5.0. Las solicitaciones sismicas de DISENO de los elementos = (analisis elastico)/R; las derivas se verifican con las fuerzas sin reducir (A.6).</t>
         </is>
       </c>
-    </row>
-    <row r="48"/>
+      <c r="C47" s="16" t="n"/>
+      <c r="D47" s="16" t="n"/>
+      <c r="E47" s="16" t="n"/>
+      <c r="F47" s="16" t="n"/>
+      <c r="G47" s="16" t="n"/>
+      <c r="H47" s="16" t="n"/>
+      <c r="I47" s="16" t="n"/>
+      <c r="J47" s="17" t="n"/>
+    </row>
+    <row r="48">
+      <c r="B48" s="20" t="n"/>
+      <c r="C48" s="21" t="n"/>
+      <c r="D48" s="21" t="n"/>
+      <c r="E48" s="21" t="n"/>
+      <c r="F48" s="21" t="n"/>
+      <c r="G48" s="21" t="n"/>
+      <c r="H48" s="21" t="n"/>
+      <c r="I48" s="21" t="n"/>
+      <c r="J48" s="22" t="n"/>
+    </row>
     <row r="50">
       <c r="B50" s="2" t="inlineStr">
         <is>
@@ -1633,1022 +1780,668 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:J80"/>
+  <dimension ref="B2:O25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="46" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="2">
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>DISENO DE VIGAS DE CARGA  (VC 40x30) - NSR-10 / ACI 318 (DMO)</t>
+      <c r="B2" s="23" t="inlineStr">
+        <is>
+          <t>CUADRO DE VIGAS Y RIOSTRAS POR TIPOS  (NSR-10/ACI - sismo / R=5)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>1. DATOS Y GEOMETRIA</t>
-        </is>
-      </c>
-      <c r="J4" s="7" t="inlineStr">
-        <is>
-          <t>Celdas azules = entrada</t>
-        </is>
-      </c>
+      <c r="B4" s="24" t="inlineStr">
+        <is>
+          <t>Materiales y refuerzo (comunes)</t>
+        </is>
+      </c>
+      <c r="C4" s="25" t="n"/>
+      <c r="D4" s="25" t="n"/>
+      <c r="E4" s="26" t="n"/>
     </row>
     <row r="5">
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>f'c</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="n">
+      <c r="B5" s="27" t="inlineStr">
+        <is>
+          <t>f'c [MPa]</t>
+        </is>
+      </c>
+      <c r="C5" s="28" t="n">
         <v>28</v>
       </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>MPa</t>
-        </is>
-      </c>
-      <c r="J5" s="7" t="inlineStr">
-        <is>
-          <t>phi=0.90 flexion - phi=0.75 cortante y torsion - rho_max(DMO)=0.025</t>
+      <c r="D5" s="27" t="inlineStr">
+        <is>
+          <t>fy [MPa]</t>
+        </is>
+      </c>
+      <c r="E5" s="28" t="n">
+        <v>420</v>
+      </c>
+      <c r="F5" s="27" t="inlineStr">
+        <is>
+          <t>recubr [m]</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="H5" s="27" t="inlineStr">
+        <is>
+          <t>Diam barra</t>
+        </is>
+      </c>
+      <c r="I5" s="28" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="J5" s="27" t="inlineStr">
+        <is>
+          <t>#5  Area-&gt;</t>
+        </is>
+      </c>
+      <c r="K5" s="28" t="n">
+        <v>199</v>
+      </c>
+      <c r="L5" s="27" t="inlineStr">
+        <is>
+          <t>mm2</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>fy = fyt</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="n">
-        <v>420</v>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>MPa</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>b (ancho)</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="n">
+      <c r="B6" s="27" t="inlineStr">
+        <is>
+          <t>Diam estribo</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="D6" s="27" t="inlineStr">
+        <is>
+          <t>#3  Av [mm2]</t>
+        </is>
+      </c>
+      <c r="F6" s="28" t="n">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Las vigas se agrupan por nivel de solicitacion en TIPOS; cada tipo se disena para su M- maximo de grupo. d, As y N de barras se calculan automaticamente. Celdas azules = entrada (envolvente del modelo SAP).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>VIGAS DE CARGA - VC 40x30</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="29" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C10" s="29" t="inlineStr">
+        <is>
+          <t>N vigas</t>
+        </is>
+      </c>
+      <c r="D10" s="29" t="inlineStr">
+        <is>
+          <t>b [m]</t>
+        </is>
+      </c>
+      <c r="E10" s="29" t="inlineStr">
+        <is>
+          <t>h [m]</t>
+        </is>
+      </c>
+      <c r="F10" s="29" t="inlineStr">
+        <is>
+          <t>M- [kN.m]</t>
+        </is>
+      </c>
+      <c r="G10" s="29" t="inlineStr">
+        <is>
+          <t>M+ [kN.m]</t>
+        </is>
+      </c>
+      <c r="H10" s="29" t="inlineStr">
+        <is>
+          <t>Vu [kN]</t>
+        </is>
+      </c>
+      <c r="I10" s="29" t="inlineStr">
+        <is>
+          <t>d [mm]</t>
+        </is>
+      </c>
+      <c r="J10" s="29" t="inlineStr">
+        <is>
+          <t>As- [mm2]</t>
+        </is>
+      </c>
+      <c r="K10" s="29" t="inlineStr">
+        <is>
+          <t>N #5</t>
+        </is>
+      </c>
+      <c r="L10" s="29" t="inlineStr">
+        <is>
+          <t>As+ [mm2]</t>
+        </is>
+      </c>
+      <c r="M10" s="29" t="inlineStr">
+        <is>
+          <t>N #5</t>
+        </is>
+      </c>
+      <c r="N10" s="29" t="inlineStr">
+        <is>
+          <t>s estribo [mm]</t>
+        </is>
+      </c>
+      <c r="O10" s="29" t="inlineStr">
+        <is>
+          <t>rho- check</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="30" t="inlineStr">
+        <is>
+          <t>VC-1</t>
+        </is>
+      </c>
+      <c r="C11" s="31" t="n">
+        <v>148</v>
+      </c>
+      <c r="D11" s="28" t="n">
         <v>0.3</v>
       </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>h (alto)</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="n">
+      <c r="E11" s="28" t="n">
         <v>0.4</v>
       </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>recubrimiento r</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Diam estribo</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>mm #3</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Diam barra long.</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="n">
-        <v>15.9</v>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>mm #5</t>
-        </is>
+      <c r="F11" s="28" t="n">
+        <v>77</v>
+      </c>
+      <c r="G11" s="28" t="n">
+        <v>58</v>
+      </c>
+      <c r="H11" s="28" t="n">
+        <v>70</v>
+      </c>
+      <c r="I11" s="31">
+        <f>E11*1000-$G$5*1000-$C$6-$I$5/2</f>
+        <v/>
+      </c>
+      <c r="J11" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(F11*1000000/(0.9*(D11*1000)*I11^2))/(0.85*$C$5)))*(D11*1000)*I11,MAX(0.25*SQRT($C$5)/$E$5,1.4/$E$5)*(D11*1000)*I11)</f>
+        <v/>
+      </c>
+      <c r="K11" s="33">
+        <f>ROUNDUP(J11/$K$5,0)</f>
+        <v/>
+      </c>
+      <c r="L11" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(G11*1000000/(0.9*(D11*1000)*I11^2))/(0.85*$C$5)))*(D11*1000)*I11,MAX(0.25*SQRT($C$5)/$E$5,1.4/$E$5)*(D11*1000)*I11)</f>
+        <v/>
+      </c>
+      <c r="M11" s="33">
+        <f>ROUNDUP(L11/$K$5,0)</f>
+        <v/>
+      </c>
+      <c r="N11" s="31">
+        <f>MIN(I11/4,6*$I$5,150)</f>
+        <v/>
+      </c>
+      <c r="O11" s="31">
+        <f>IF(J11/((D11*1000)*I11)&lt;=0.025,"OK","REVISAR")</f>
+        <v/>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Area barra long.</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="n">
-        <v>199</v>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
+      <c r="B12" s="30" t="inlineStr">
+        <is>
+          <t>VC-2</t>
+        </is>
+      </c>
+      <c r="C12" s="31" t="n">
+        <v>120</v>
+      </c>
+      <c r="D12" s="28" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E12" s="28" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F12" s="28" t="n">
+        <v>118</v>
+      </c>
+      <c r="G12" s="28" t="n">
+        <v>101</v>
+      </c>
+      <c r="H12" s="28" t="n">
+        <v>86</v>
+      </c>
+      <c r="I12" s="31">
+        <f>E12*1000-$G$5*1000-$C$6-$I$5/2</f>
+        <v/>
+      </c>
+      <c r="J12" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(F12*1000000/(0.9*(D12*1000)*I12^2))/(0.85*$C$5)))*(D12*1000)*I12,MAX(0.25*SQRT($C$5)/$E$5,1.4/$E$5)*(D12*1000)*I12)</f>
+        <v/>
+      </c>
+      <c r="K12" s="33">
+        <f>ROUNDUP(J12/$K$5,0)</f>
+        <v/>
+      </c>
+      <c r="L12" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(G12*1000000/(0.9*(D12*1000)*I12^2))/(0.85*$C$5)))*(D12*1000)*I12,MAX(0.25*SQRT($C$5)/$E$5,1.4/$E$5)*(D12*1000)*I12)</f>
+        <v/>
+      </c>
+      <c r="M12" s="33">
+        <f>ROUNDUP(L12/$K$5,0)</f>
+        <v/>
+      </c>
+      <c r="N12" s="31">
+        <f>MIN(I12/4,6*$I$5,150)</f>
+        <v/>
+      </c>
+      <c r="O12" s="31">
+        <f>IF(J12/((D12*1000)*I12)&lt;=0.025,"OK","REVISAR")</f>
+        <v/>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Area 2 ramas Av</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="n">
+      <c r="B13" s="30" t="inlineStr">
+        <is>
+          <t>VC-3</t>
+        </is>
+      </c>
+      <c r="C13" s="31" t="n">
+        <v>12</v>
+      </c>
+      <c r="D13" s="28" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E13" s="28" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F13" s="28" t="n">
         <v>142</v>
       </c>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Luz libre Ln</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
+      <c r="G13" s="28" t="n">
+        <v>79</v>
+      </c>
+      <c r="H13" s="28" t="n">
+        <v>108</v>
+      </c>
+      <c r="I13" s="31">
+        <f>E13*1000-$G$5*1000-$C$6-$I$5/2</f>
+        <v/>
+      </c>
+      <c r="J13" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(F13*1000000/(0.9*(D13*1000)*I13^2))/(0.85*$C$5)))*(D13*1000)*I13,MAX(0.25*SQRT($C$5)/$E$5,1.4/$E$5)*(D13*1000)*I13)</f>
+        <v/>
+      </c>
+      <c r="K13" s="33">
+        <f>ROUNDUP(J13/$K$5,0)</f>
+        <v/>
+      </c>
+      <c r="L13" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(G13*1000000/(0.9*(D13*1000)*I13^2))/(0.85*$C$5)))*(D13*1000)*I13,MAX(0.25*SQRT($C$5)/$E$5,1.4/$E$5)*(D13*1000)*I13)</f>
+        <v/>
+      </c>
+      <c r="M13" s="33">
+        <f>ROUNDUP(L13/$K$5,0)</f>
+        <v/>
+      </c>
+      <c r="N13" s="31">
+        <f>MIN(I13/4,6*$I$5,150)</f>
+        <v/>
+      </c>
+      <c r="O13" s="31">
+        <f>IF(J13/((D13*1000)*I13)&lt;=0.025,"OK","REVISAR")</f>
+        <v/>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>d = h - r - est - bl/2</t>
-        </is>
-      </c>
-      <c r="C15" s="14">
-        <f>C8*1000-C9*1000-C10-C11/2</f>
-        <v/>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>mm</t>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>RIOSTRAS / VIGAS DE RIGIDEZ - VR 40x35</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="29" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C16" s="29" t="inlineStr">
+        <is>
+          <t>N vigas</t>
+        </is>
+      </c>
+      <c r="D16" s="29" t="inlineStr">
+        <is>
+          <t>b [m]</t>
+        </is>
+      </c>
+      <c r="E16" s="29" t="inlineStr">
+        <is>
+          <t>h [m]</t>
+        </is>
+      </c>
+      <c r="F16" s="29" t="inlineStr">
+        <is>
+          <t>M- [kN.m]</t>
+        </is>
+      </c>
+      <c r="G16" s="29" t="inlineStr">
+        <is>
+          <t>M+ [kN.m]</t>
+        </is>
+      </c>
+      <c r="H16" s="29" t="inlineStr">
+        <is>
+          <t>Vu [kN]</t>
+        </is>
+      </c>
+      <c r="I16" s="29" t="inlineStr">
+        <is>
+          <t>d [mm]</t>
+        </is>
+      </c>
+      <c r="J16" s="29" t="inlineStr">
+        <is>
+          <t>As- [mm2]</t>
+        </is>
+      </c>
+      <c r="K16" s="29" t="inlineStr">
+        <is>
+          <t>N #5</t>
+        </is>
+      </c>
+      <c r="L16" s="29" t="inlineStr">
+        <is>
+          <t>As+ [mm2]</t>
+        </is>
+      </c>
+      <c r="M16" s="29" t="inlineStr">
+        <is>
+          <t>N #5</t>
+        </is>
+      </c>
+      <c r="N16" s="29" t="inlineStr">
+        <is>
+          <t>s estribo [mm]</t>
+        </is>
+      </c>
+      <c r="O16" s="29" t="inlineStr">
+        <is>
+          <t>rho- check</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>2. SOLICITACIONES (envolvente SAP, sismo / R=5)</t>
-        </is>
+      <c r="B17" s="30" t="inlineStr">
+        <is>
+          <t>VR-1</t>
+        </is>
+      </c>
+      <c r="C17" s="31" t="n">
+        <v>170</v>
+      </c>
+      <c r="D17" s="28" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="E17" s="28" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F17" s="28" t="n">
+        <v>100</v>
+      </c>
+      <c r="G17" s="28" t="n">
+        <v>74</v>
+      </c>
+      <c r="H17" s="28" t="n">
+        <v>104</v>
+      </c>
+      <c r="I17" s="31">
+        <f>E17*1000-$G$5*1000-$C$6-$I$5/2</f>
+        <v/>
+      </c>
+      <c r="J17" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(F17*1000000/(0.9*(D17*1000)*I17^2))/(0.85*$C$5)))*(D17*1000)*I17,MAX(0.25*SQRT($C$5)/$E$5,1.4/$E$5)*(D17*1000)*I17)</f>
+        <v/>
+      </c>
+      <c r="K17" s="33">
+        <f>ROUNDUP(J17/$K$5,0)</f>
+        <v/>
+      </c>
+      <c r="L17" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(G17*1000000/(0.9*(D17*1000)*I17^2))/(0.85*$C$5)))*(D17*1000)*I17,MAX(0.25*SQRT($C$5)/$E$5,1.4/$E$5)*(D17*1000)*I17)</f>
+        <v/>
+      </c>
+      <c r="M17" s="33">
+        <f>ROUNDUP(L17/$K$5,0)</f>
+        <v/>
+      </c>
+      <c r="N17" s="31">
+        <f>MIN(I17/4,6*$I$5,150)</f>
+        <v/>
+      </c>
+      <c r="O17" s="31">
+        <f>IF(J17/((D17*1000)*I17)&lt;=0.025,"OK","REVISAR")</f>
+        <v/>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Mu (-) negativo</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="n">
-        <v>142</v>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>kN.m</t>
-        </is>
+      <c r="B18" s="30" t="inlineStr">
+        <is>
+          <t>VR-2</t>
+        </is>
+      </c>
+      <c r="C18" s="31" t="n">
+        <v>120</v>
+      </c>
+      <c r="D18" s="28" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="E18" s="28" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F18" s="28" t="n">
+        <v>135</v>
+      </c>
+      <c r="G18" s="28" t="n">
+        <v>98</v>
+      </c>
+      <c r="H18" s="28" t="n">
+        <v>133</v>
+      </c>
+      <c r="I18" s="31">
+        <f>E18*1000-$G$5*1000-$C$6-$I$5/2</f>
+        <v/>
+      </c>
+      <c r="J18" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(F18*1000000/(0.9*(D18*1000)*I18^2))/(0.85*$C$5)))*(D18*1000)*I18,MAX(0.25*SQRT($C$5)/$E$5,1.4/$E$5)*(D18*1000)*I18)</f>
+        <v/>
+      </c>
+      <c r="K18" s="33">
+        <f>ROUNDUP(J18/$K$5,0)</f>
+        <v/>
+      </c>
+      <c r="L18" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(G18*1000000/(0.9*(D18*1000)*I18^2))/(0.85*$C$5)))*(D18*1000)*I18,MAX(0.25*SQRT($C$5)/$E$5,1.4/$E$5)*(D18*1000)*I18)</f>
+        <v/>
+      </c>
+      <c r="M18" s="33">
+        <f>ROUNDUP(L18/$K$5,0)</f>
+        <v/>
+      </c>
+      <c r="N18" s="31">
+        <f>MIN(I18/4,6*$I$5,150)</f>
+        <v/>
+      </c>
+      <c r="O18" s="31">
+        <f>IF(J18/((D18*1000)*I18)&lt;=0.025,"OK","REVISAR")</f>
+        <v/>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Mu (+) positivo</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="n">
-        <v>101</v>
-      </c>
-      <c r="D19" s="9" t="inlineStr">
-        <is>
-          <t>kN.m</t>
-        </is>
+      <c r="B19" s="30" t="inlineStr">
+        <is>
+          <t>VR-3</t>
+        </is>
+      </c>
+      <c r="C19" s="31" t="n">
+        <v>6</v>
+      </c>
+      <c r="D19" s="28" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="E19" s="28" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F19" s="28" t="n">
+        <v>186</v>
+      </c>
+      <c r="G19" s="28" t="n">
+        <v>138</v>
+      </c>
+      <c r="H19" s="28" t="n">
+        <v>189</v>
+      </c>
+      <c r="I19" s="31">
+        <f>E19*1000-$G$5*1000-$C$6-$I$5/2</f>
+        <v/>
+      </c>
+      <c r="J19" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(F19*1000000/(0.9*(D19*1000)*I19^2))/(0.85*$C$5)))*(D19*1000)*I19,MAX(0.25*SQRT($C$5)/$E$5,1.4/$E$5)*(D19*1000)*I19)</f>
+        <v/>
+      </c>
+      <c r="K19" s="33">
+        <f>ROUNDUP(J19/$K$5,0)</f>
+        <v/>
+      </c>
+      <c r="L19" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(G19*1000000/(0.9*(D19*1000)*I19^2))/(0.85*$C$5)))*(D19*1000)*I19,MAX(0.25*SQRT($C$5)/$E$5,1.4/$E$5)*(D19*1000)*I19)</f>
+        <v/>
+      </c>
+      <c r="M19" s="33">
+        <f>ROUNDUP(L19/$K$5,0)</f>
+        <v/>
+      </c>
+      <c r="N19" s="31">
+        <f>MIN(I19/4,6*$I$5,150)</f>
+        <v/>
+      </c>
+      <c r="O19" s="31">
+        <f>IF(J19/((D19*1000)*I19)&lt;=0.025,"OK","REVISAR")</f>
+        <v/>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>Vu cortante</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="n">
-        <v>108</v>
-      </c>
-      <c r="D20" s="9" t="inlineStr">
-        <is>
-          <t>kN</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Tu torsion</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="n">
-        <v>20</v>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
-        <is>
-          <t>kN.m</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>3. FLEXION - Momento NEGATIVO (acero superior)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>Rn = Mu/(phi b d2)</t>
-        </is>
-      </c>
-      <c r="C24" s="9">
-        <f>C18*1000000/(0.9*(C7*1000)*C15^2)</f>
-        <v/>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>MPa</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>rho requerido</t>
-        </is>
-      </c>
-      <c r="C25" s="9">
-        <f>(0.85*C5/C6)*(1-SQRT(1-2*C24/(0.85*C5)))</f>
-        <v/>
-      </c>
-      <c r="D25" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>As requerido</t>
-        </is>
-      </c>
-      <c r="C26" s="9">
-        <f>C25*(C7*1000)*C15</f>
-        <v/>
-      </c>
-      <c r="D26" s="9" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>As minimo (C.10.5)</t>
-        </is>
-      </c>
-      <c r="C27" s="9">
-        <f>MAX(0.25*SQRT(C5)/C6,1.4/C6)*(C7*1000)*C15</f>
-        <v/>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>As maximo (rho=0.025)</t>
-        </is>
-      </c>
-      <c r="C28" s="9">
-        <f>0.025*(C7*1000)*C15</f>
-        <v/>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>As de diseno</t>
-        </is>
-      </c>
-      <c r="C29" s="15">
-        <f>MAX(C26,C27)</f>
-        <v/>
-      </c>
-      <c r="D29" s="9" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>N barras</t>
-        </is>
-      </c>
-      <c r="C30" s="14">
-        <f>ROUNDUP(C29/C12,0)</f>
-        <v/>
-      </c>
-      <c r="D30" s="9" t="inlineStr">
-        <is>
-          <t>u</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>As colocado</t>
-        </is>
-      </c>
-      <c r="C31" s="15">
-        <f>C30*C12</f>
-        <v/>
-      </c>
-      <c r="D31" s="9" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>a (bloque comp.)</t>
-        </is>
-      </c>
-      <c r="C32" s="9">
-        <f>C31*C6/(0.85*C5*(C7*1000))</f>
-        <v/>
-      </c>
-      <c r="D32" s="9" t="inlineStr">
-        <is>
-          <t>mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>phiMn</t>
-        </is>
-      </c>
-      <c r="C33" s="14">
-        <f>0.9*C31*C6*(C15-C32/2)/1000000</f>
-        <v/>
-      </c>
-      <c r="D33" s="9" t="inlineStr">
-        <is>
-          <t>kN.m</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="6" t="inlineStr">
-        <is>
-          <t>VERIFICACION flexion (-)</t>
-        </is>
-      </c>
-      <c r="C34" s="11">
-        <f>IF(AND(C33&gt;=C18,C29&lt;=C28,C29&gt;=C27),"CUMPLE","REVISAR")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>4. FLEXION - Momento POSITIVO (acero inferior)</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>Rn</t>
-        </is>
-      </c>
-      <c r="C37" s="9">
-        <f>C19*1000000/(0.9*(C7*1000)*C15^2)</f>
-        <v/>
-      </c>
-      <c r="D37" s="9" t="inlineStr">
-        <is>
-          <t>MPa</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>rho requerido</t>
-        </is>
-      </c>
-      <c r="C38" s="9">
-        <f>(0.85*C5/C6)*(1-SQRT(1-2*C37/(0.85*C5)))</f>
-        <v/>
-      </c>
-      <c r="D38" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>As requerido</t>
-        </is>
-      </c>
-      <c r="C39" s="9">
-        <f>C38*(C7*1000)*C15</f>
-        <v/>
-      </c>
-      <c r="D39" s="9" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>As de diseno (&gt;= As min)</t>
-        </is>
-      </c>
-      <c r="C40" s="15">
-        <f>MAX(C39,C27)</f>
-        <v/>
-      </c>
-      <c r="D40" s="9" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>N barras</t>
-        </is>
-      </c>
-      <c r="C41" s="14">
-        <f>ROUNDUP(C40/C12,0)</f>
-        <v/>
-      </c>
-      <c r="D41" s="9" t="inlineStr">
-        <is>
-          <t>u</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>As colocado</t>
-        </is>
-      </c>
-      <c r="C42" s="15">
-        <f>C41*C12</f>
-        <v/>
-      </c>
-      <c r="D42" s="9" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="B43" s="4" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="C43" s="9">
-        <f>C42*C6/(0.85*C5*(C7*1000))</f>
-        <v/>
-      </c>
-      <c r="D43" s="9" t="inlineStr">
-        <is>
-          <t>mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="B44" s="4" t="inlineStr">
-        <is>
-          <t>phiMn</t>
-        </is>
-      </c>
-      <c r="C44" s="14">
-        <f>0.9*C42*C6*(C15-C43/2)/1000000</f>
-        <v/>
-      </c>
-      <c r="D44" s="9" t="inlineStr">
-        <is>
-          <t>kN.m</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="B45" s="6" t="inlineStr">
-        <is>
-          <t>VERIFICACION flexion (+)</t>
-        </is>
-      </c>
-      <c r="C45" s="11">
-        <f>IF(C44&gt;=C19,"CUMPLE","REVISAR")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>5. CORTANTE  (phi=0.75)</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="B48" s="4" t="inlineStr">
-        <is>
-          <t>Vc = 0.17 raiz(f'c) b d</t>
-        </is>
-      </c>
-      <c r="C48" s="9">
-        <f>0.17*SQRT(C5)*(C7*1000)*C15/1000</f>
-        <v/>
-      </c>
-      <c r="D48" s="9" t="inlineStr">
-        <is>
-          <t>kN</t>
-        </is>
-      </c>
-      <c r="J48" s="7" t="inlineStr">
-        <is>
-          <t>Estribos #3 de 2 ramas. Confinamiento = 2h desde cada cara del nudo (DMO C.21.3.4).</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="B49" s="4" t="inlineStr">
-        <is>
-          <t>phiVc</t>
-        </is>
-      </c>
-      <c r="C49" s="9">
-        <f>0.75*C48</f>
-        <v/>
-      </c>
-      <c r="D49" s="9" t="inlineStr">
-        <is>
-          <t>kN</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="B50" s="4" t="inlineStr">
-        <is>
-          <t>Vs requerido = Vu/phi - Vc</t>
-        </is>
-      </c>
-      <c r="C50" s="9">
-        <f>MAX(C20/0.75-C48,0)</f>
-        <v/>
-      </c>
-      <c r="D50" s="9" t="inlineStr">
-        <is>
-          <t>kN</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="B51" s="4" t="inlineStr">
-        <is>
-          <t>Vs max = 0.66 raiz(f'c) b d</t>
-        </is>
-      </c>
-      <c r="C51" s="9">
-        <f>0.66*SQRT(C5)*(C7*1000)*C15/1000</f>
-        <v/>
-      </c>
-      <c r="D51" s="9" t="inlineStr">
-        <is>
-          <t>kN</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="B52" s="4" t="inlineStr">
-        <is>
-          <t>s requerido = Av fyt d/Vs</t>
-        </is>
-      </c>
-      <c r="C52" s="9">
-        <f>IF(C50&gt;0,C13*C6*C15/(C50*1000),300)</f>
-        <v/>
-      </c>
-      <c r="D52" s="9" t="inlineStr">
-        <is>
-          <t>mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="B53" s="4" t="inlineStr">
-        <is>
-          <t>s max confinamiento DMO</t>
-        </is>
-      </c>
-      <c r="C53" s="9">
-        <f>MIN(C15/4,6*C11,150)</f>
-        <v/>
-      </c>
-      <c r="D53" s="9" t="inlineStr">
-        <is>
-          <t>mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="B54" s="4" t="inlineStr">
-        <is>
-          <t>Separacion a adoptar</t>
-        </is>
-      </c>
-      <c r="C54" s="14">
-        <f>IF(C50&gt;0,MIN(C52,C53),C53)</f>
-        <v/>
-      </c>
-      <c r="D54" s="9" t="inlineStr">
-        <is>
-          <t>mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="B55" s="6" t="inlineStr">
-        <is>
-          <t>VERIFICACION cortante</t>
-        </is>
-      </c>
-      <c r="C55" s="11">
-        <f>IF(C50&lt;=C51,"CUMPLE (seccion OK)","AUMENTAR SECCION")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57">
-      <c r="B57" s="2" t="inlineStr">
-        <is>
-          <t>6. CORTANTE POR CAPACIDAD (DMO C.21.3.4.2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="B58" s="4" t="inlineStr">
-        <is>
-          <t>Mpr(-) = 1.25 As fy (d-a/2)</t>
-        </is>
-      </c>
-      <c r="C58" s="9">
-        <f>1.25*C31*C6*(C15-(1.25*C31*C6/(0.85*C5*(C7*1000)))/2)/1000000</f>
-        <v/>
-      </c>
-      <c r="D58" s="9" t="inlineStr">
-        <is>
-          <t>kN.m</t>
-        </is>
-      </c>
-      <c r="J58" s="7" t="inlineStr">
-        <is>
-          <t>Sumar el cortante gravitacional del tramo a Ve. Gobierna el mayor entre Vu y Ve.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="B59" s="4" t="inlineStr">
-        <is>
-          <t>Mpr(+)</t>
-        </is>
-      </c>
-      <c r="C59" s="9">
-        <f>1.25*C42*C6*(C15-(1.25*C42*C6/(0.85*C5*(C7*1000)))/2)/1000000</f>
-        <v/>
-      </c>
-      <c r="D59" s="9" t="inlineStr">
-        <is>
-          <t>kN.m</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="B60" s="4" t="inlineStr">
-        <is>
-          <t>Ve = (Mpr- + Mpr+)/Ln</t>
-        </is>
-      </c>
-      <c r="C60" s="9">
-        <f>(C58+C59)/C14</f>
-        <v/>
-      </c>
-      <c r="D60" s="9" t="inlineStr">
-        <is>
-          <t>kN</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="B61" s="4" t="inlineStr">
-        <is>
-          <t>V de diseno = max(Vu, Ve)</t>
-        </is>
-      </c>
-      <c r="C61" s="14">
-        <f>MAX(C20,C60)</f>
-        <v/>
-      </c>
-      <c r="D61" s="9" t="inlineStr">
-        <is>
-          <t>kN</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="B63" s="2" t="inlineStr">
-        <is>
-          <t>7. TORSION  (phi=0.75, theta=45)</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="B64" s="4" t="inlineStr">
-        <is>
-          <t>Acp = b h</t>
-        </is>
-      </c>
-      <c r="C64" s="9">
-        <f>(C7*1000)*(C8*1000)</f>
-        <v/>
-      </c>
-      <c r="D64" s="9" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-      <c r="J64" s="7" t="inlineStr">
-        <is>
-          <t>Estribo total = Av/s(cortante) + 2(At/s). Al se reparte en el perimetro.</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="B65" s="4" t="inlineStr">
-        <is>
-          <t>pcp = 2(b+h)</t>
-        </is>
-      </c>
-      <c r="C65" s="9">
-        <f>2*((C7*1000)+(C8*1000))</f>
-        <v/>
-      </c>
-      <c r="D65" s="9" t="inlineStr">
-        <is>
-          <t>mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="B66" s="4" t="inlineStr">
-        <is>
-          <t>T umbral = phi 0.083 raiz(f'c) Acp2/pcp</t>
-        </is>
-      </c>
-      <c r="C66" s="9">
-        <f>0.75*0.083*SQRT(C5)*(C64^2/C65)/1000000</f>
-        <v/>
-      </c>
-      <c r="D66" s="9" t="inlineStr">
-        <is>
-          <t>kN.m</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="B67" s="4" t="inlineStr">
-        <is>
-          <t>Requiere torsion?</t>
-        </is>
-      </c>
-      <c r="C67" s="14">
-        <f>IF(C21&gt;C66,"SI - disenar","No - despreciable")</f>
-        <v/>
-      </c>
-      <c r="D67" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="B68" s="4" t="inlineStr">
-        <is>
-          <t>Aoh = (b-2r)(h-2r)</t>
-        </is>
-      </c>
-      <c r="C68" s="9">
-        <f>((C7*1000)-2*C9*1000)*((C8*1000)-2*C9*1000)</f>
-        <v/>
-      </c>
-      <c r="D68" s="9" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="B69" s="4" t="inlineStr">
-        <is>
-          <t>ph = 2[(b-2r)+(h-2r)]</t>
-        </is>
-      </c>
-      <c r="C69" s="9">
-        <f>2*(((C7*1000)-2*C9*1000)+((C8*1000)-2*C9*1000))</f>
-        <v/>
-      </c>
-      <c r="D69" s="9" t="inlineStr">
-        <is>
-          <t>mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="B70" s="4" t="inlineStr">
-        <is>
-          <t>Ao = 0.85 Aoh</t>
-        </is>
-      </c>
-      <c r="C70" s="9">
-        <f>0.85*C68</f>
-        <v/>
-      </c>
-      <c r="D70" s="9" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="B71" s="4" t="inlineStr">
-        <is>
-          <t>At/s (estribo torsion)</t>
-        </is>
-      </c>
-      <c r="C71" s="15">
-        <f>IF(C21&gt;C66,C21*1000000/(0.75*2*C70*C6),0)</f>
-        <v/>
-      </c>
-      <c r="D71" s="9" t="inlineStr">
-        <is>
-          <t>mm2/mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="B72" s="4" t="inlineStr">
-        <is>
-          <t>Al (long. por torsion)</t>
-        </is>
-      </c>
-      <c r="C72" s="15">
-        <f>IF(C21&gt;C66,C71*C69,0)</f>
-        <v/>
-      </c>
-      <c r="D72" s="9" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="B74" s="2" t="inlineStr">
-        <is>
-          <t>8. DEFLEXION (C.9.5)</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="B75" s="4" t="inlineStr">
-        <is>
-          <t>h min = Ln/18.5</t>
-        </is>
-      </c>
-      <c r="C75" s="9">
-        <f>C14/18.5</f>
-        <v/>
-      </c>
-      <c r="D75" s="9" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="B76" s="6" t="inlineStr">
-        <is>
-          <t>VERIFICACION</t>
-        </is>
-      </c>
-      <c r="C76" s="11">
-        <f>IF(C8&gt;=C75,"CUMPLE","REVISAR")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="78">
-      <c r="B78" s="2" t="inlineStr">
-        <is>
-          <t>9. DESPIECE (resumen)</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="40" customHeight="1">
-      <c r="B79" s="7" t="inlineStr">
-        <is>
-          <t>Acero superior: As(-) corrido + bastones en zona negativa (Ln/4 + ld). Inferior: As(+) corrido. Estribos #3: confinamiento @ s_adoptar en 2h desde cada cara, resto @ d/2. Ganchos sismicos 135 grados.</t>
-        </is>
-      </c>
-    </row>
-    <row r="80"/>
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>VR-4</t>
+        </is>
+      </c>
+      <c r="C20" s="31" t="n">
+        <v>14</v>
+      </c>
+      <c r="D20" s="28" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="E20" s="28" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F20" s="28" t="n">
+        <v>243</v>
+      </c>
+      <c r="G20" s="28" t="n">
+        <v>134</v>
+      </c>
+      <c r="H20" s="28" t="n">
+        <v>202</v>
+      </c>
+      <c r="I20" s="31">
+        <f>E20*1000-$G$5*1000-$C$6-$I$5/2</f>
+        <v/>
+      </c>
+      <c r="J20" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(F20*1000000/(0.9*(D20*1000)*I20^2))/(0.85*$C$5)))*(D20*1000)*I20,MAX(0.25*SQRT($C$5)/$E$5,1.4/$E$5)*(D20*1000)*I20)</f>
+        <v/>
+      </c>
+      <c r="K20" s="33">
+        <f>ROUNDUP(J20/$K$5,0)</f>
+        <v/>
+      </c>
+      <c r="L20" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(G20*1000000/(0.9*(D20*1000)*I20^2))/(0.85*$C$5)))*(D20*1000)*I20,MAX(0.25*SQRT($C$5)/$E$5,1.4/$E$5)*(D20*1000)*I20)</f>
+        <v/>
+      </c>
+      <c r="M20" s="33">
+        <f>ROUNDUP(L20/$K$5,0)</f>
+        <v/>
+      </c>
+      <c r="N20" s="31">
+        <f>MIN(I20/4,6*$I$5,150)</f>
+        <v/>
+      </c>
+      <c r="O20" s="31">
+        <f>IF(J20/((D20*1000)*I20)&lt;=0.025,"OK","REVISAR")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="46" customHeight="1">
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Cada tipo agrupa las vigas con M- hasta el valor indicado. El N de barras es para flexion; en apoyos se coloca As- (bastones Ln/4+ld) y en el centro As+ corrido. Estribos #3 @ s en zona de confinamiento (2h desde la cara del nudo) y @ d/2 en el resto. Torsion y cortante por capacidad: ver hojas 'Diseno Vigas' y 'Diseno Riostras' (calculo detallado del tipo critico VC-3 y VR-4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24"/>
+    <row r="25"/>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B79:J80"/>
-    <mergeCell ref="B2:J2"/>
+  <mergeCells count="6">
+    <mergeCell ref="B9:O9"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B2:O2"/>
+    <mergeCell ref="B15:O15"/>
+    <mergeCell ref="B7:O7"/>
+    <mergeCell ref="B23:O25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2678,7 +2471,7 @@
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>DISENO DE RIOSTRAS / VIGAS DE RIGIDEZ  (VR 40x35) - NSR-10 / ACI 318 (DMO)</t>
+          <t>DISENO DE VIGAS DE CARGA  (VC 40x30) - NSR-10 / ACI 318 (DMO)</t>
         </is>
       </c>
     </row>
@@ -2736,7 +2529,7 @@
         </is>
       </c>
       <c r="C7" s="5" t="n">
-        <v>0.35</v>
+        <v>0.3</v>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
@@ -2841,7 +2634,7 @@
         </is>
       </c>
       <c r="C14" s="5" t="n">
-        <v>5.1</v>
+        <v>4.9</v>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
@@ -2879,7 +2672,7 @@
         </is>
       </c>
       <c r="C18" s="5" t="n">
-        <v>250</v>
+        <v>142</v>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
@@ -2894,7 +2687,7 @@
         </is>
       </c>
       <c r="C19" s="5" t="n">
-        <v>138</v>
+        <v>101</v>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
@@ -2909,7 +2702,7 @@
         </is>
       </c>
       <c r="C20" s="5" t="n">
-        <v>202</v>
+        <v>108</v>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
@@ -2924,7 +2717,7 @@
         </is>
       </c>
       <c r="C21" s="5" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
@@ -3682,6 +3475,1033 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:J80"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="46" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>DISENO DE RIOSTRAS / VIGAS DE RIGIDEZ  (VR 40x35) - NSR-10 / ACI 318 (DMO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>1. DATOS Y GEOMETRIA</t>
+        </is>
+      </c>
+      <c r="J4" s="7" t="inlineStr">
+        <is>
+          <t>Celdas azules = entrada</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>f'c</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>phi=0.90 flexion - phi=0.75 cortante y torsion - rho_max(DMO)=0.025</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>fy = fyt</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>420</v>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>b (ancho)</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>h (alto)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>recubrimiento r</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Diam estribo</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>mm #3</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Diam barra long.</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>mm #5</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Area barra long.</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>199</v>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Area 2 ramas Av</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>142</v>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Luz libre Ln</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>d = h - r - est - bl/2</t>
+        </is>
+      </c>
+      <c r="C15" s="14">
+        <f>C8*1000-C9*1000-C10-C11/2</f>
+        <v/>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>2. SOLICITACIONES (envolvente SAP, sismo / R=5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Mu (-) negativo</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>250</v>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>kN.m</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Mu (+) positivo</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>138</v>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>kN.m</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Vu cortante</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>202</v>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>kN</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Tu torsion</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>kN.m</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>3. FLEXION - Momento NEGATIVO (acero superior)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Rn = Mu/(phi b d2)</t>
+        </is>
+      </c>
+      <c r="C24" s="9">
+        <f>C18*1000000/(0.9*(C7*1000)*C15^2)</f>
+        <v/>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>rho requerido</t>
+        </is>
+      </c>
+      <c r="C25" s="9">
+        <f>(0.85*C5/C6)*(1-SQRT(1-2*C24/(0.85*C5)))</f>
+        <v/>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>As requerido</t>
+        </is>
+      </c>
+      <c r="C26" s="9">
+        <f>C25*(C7*1000)*C15</f>
+        <v/>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>As minimo (C.10.5)</t>
+        </is>
+      </c>
+      <c r="C27" s="9">
+        <f>MAX(0.25*SQRT(C5)/C6,1.4/C6)*(C7*1000)*C15</f>
+        <v/>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>As maximo (rho=0.025)</t>
+        </is>
+      </c>
+      <c r="C28" s="9">
+        <f>0.025*(C7*1000)*C15</f>
+        <v/>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>As de diseno</t>
+        </is>
+      </c>
+      <c r="C29" s="15">
+        <f>MAX(C26,C27)</f>
+        <v/>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>N barras</t>
+        </is>
+      </c>
+      <c r="C30" s="14">
+        <f>ROUNDUP(C29/C12,0)</f>
+        <v/>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>u</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>As colocado</t>
+        </is>
+      </c>
+      <c r="C31" s="15">
+        <f>C30*C12</f>
+        <v/>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>a (bloque comp.)</t>
+        </is>
+      </c>
+      <c r="C32" s="9">
+        <f>C31*C6/(0.85*C5*(C7*1000))</f>
+        <v/>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>phiMn</t>
+        </is>
+      </c>
+      <c r="C33" s="14">
+        <f>0.9*C31*C6*(C15-C32/2)/1000000</f>
+        <v/>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>kN.m</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>VERIFICACION flexion (-)</t>
+        </is>
+      </c>
+      <c r="C34" s="11">
+        <f>IF(AND(C33&gt;=C18,C29&lt;=C28,C29&gt;=C27),"CUMPLE","REVISAR")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>4. FLEXION - Momento POSITIVO (acero inferior)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Rn</t>
+        </is>
+      </c>
+      <c r="C37" s="9">
+        <f>C19*1000000/(0.9*(C7*1000)*C15^2)</f>
+        <v/>
+      </c>
+      <c r="D37" s="9" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>rho requerido</t>
+        </is>
+      </c>
+      <c r="C38" s="9">
+        <f>(0.85*C5/C6)*(1-SQRT(1-2*C37/(0.85*C5)))</f>
+        <v/>
+      </c>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>As requerido</t>
+        </is>
+      </c>
+      <c r="C39" s="9">
+        <f>C38*(C7*1000)*C15</f>
+        <v/>
+      </c>
+      <c r="D39" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>As de diseno (&gt;= As min)</t>
+        </is>
+      </c>
+      <c r="C40" s="15">
+        <f>MAX(C39,C27)</f>
+        <v/>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>N barras</t>
+        </is>
+      </c>
+      <c r="C41" s="14">
+        <f>ROUNDUP(C40/C12,0)</f>
+        <v/>
+      </c>
+      <c r="D41" s="9" t="inlineStr">
+        <is>
+          <t>u</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>As colocado</t>
+        </is>
+      </c>
+      <c r="C42" s="15">
+        <f>C41*C12</f>
+        <v/>
+      </c>
+      <c r="D42" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="C43" s="9">
+        <f>C42*C6/(0.85*C5*(C7*1000))</f>
+        <v/>
+      </c>
+      <c r="D43" s="9" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>phiMn</t>
+        </is>
+      </c>
+      <c r="C44" s="14">
+        <f>0.9*C42*C6*(C15-C43/2)/1000000</f>
+        <v/>
+      </c>
+      <c r="D44" s="9" t="inlineStr">
+        <is>
+          <t>kN.m</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>VERIFICACION flexion (+)</t>
+        </is>
+      </c>
+      <c r="C45" s="11">
+        <f>IF(C44&gt;=C19,"CUMPLE","REVISAR")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>5. CORTANTE  (phi=0.75)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Vc = 0.17 raiz(f'c) b d</t>
+        </is>
+      </c>
+      <c r="C48" s="9">
+        <f>0.17*SQRT(C5)*(C7*1000)*C15/1000</f>
+        <v/>
+      </c>
+      <c r="D48" s="9" t="inlineStr">
+        <is>
+          <t>kN</t>
+        </is>
+      </c>
+      <c r="J48" s="7" t="inlineStr">
+        <is>
+          <t>Estribos #3 de 2 ramas. Confinamiento = 2h desde cada cara del nudo (DMO C.21.3.4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>phiVc</t>
+        </is>
+      </c>
+      <c r="C49" s="9">
+        <f>0.75*C48</f>
+        <v/>
+      </c>
+      <c r="D49" s="9" t="inlineStr">
+        <is>
+          <t>kN</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Vs requerido = Vu/phi - Vc</t>
+        </is>
+      </c>
+      <c r="C50" s="9">
+        <f>MAX(C20/0.75-C48,0)</f>
+        <v/>
+      </c>
+      <c r="D50" s="9" t="inlineStr">
+        <is>
+          <t>kN</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Vs max = 0.66 raiz(f'c) b d</t>
+        </is>
+      </c>
+      <c r="C51" s="9">
+        <f>0.66*SQRT(C5)*(C7*1000)*C15/1000</f>
+        <v/>
+      </c>
+      <c r="D51" s="9" t="inlineStr">
+        <is>
+          <t>kN</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>s requerido = Av fyt d/Vs</t>
+        </is>
+      </c>
+      <c r="C52" s="9">
+        <f>IF(C50&gt;0,C13*C6*C15/(C50*1000),300)</f>
+        <v/>
+      </c>
+      <c r="D52" s="9" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>s max confinamiento DMO</t>
+        </is>
+      </c>
+      <c r="C53" s="9">
+        <f>MIN(C15/4,6*C11,150)</f>
+        <v/>
+      </c>
+      <c r="D53" s="9" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>Separacion a adoptar</t>
+        </is>
+      </c>
+      <c r="C54" s="14">
+        <f>IF(C50&gt;0,MIN(C52,C53),C53)</f>
+        <v/>
+      </c>
+      <c r="D54" s="9" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>VERIFICACION cortante</t>
+        </is>
+      </c>
+      <c r="C55" s="11">
+        <f>IF(C50&lt;=C51,"CUMPLE (seccion OK)","AUMENTAR SECCION")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>6. CORTANTE POR CAPACIDAD (DMO C.21.3.4.2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>Mpr(-) = 1.25 As fy (d-a/2)</t>
+        </is>
+      </c>
+      <c r="C58" s="9">
+        <f>1.25*C31*C6*(C15-(1.25*C31*C6/(0.85*C5*(C7*1000)))/2)/1000000</f>
+        <v/>
+      </c>
+      <c r="D58" s="9" t="inlineStr">
+        <is>
+          <t>kN.m</t>
+        </is>
+      </c>
+      <c r="J58" s="7" t="inlineStr">
+        <is>
+          <t>Sumar el cortante gravitacional del tramo a Ve. Gobierna el mayor entre Vu y Ve.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>Mpr(+)</t>
+        </is>
+      </c>
+      <c r="C59" s="9">
+        <f>1.25*C42*C6*(C15-(1.25*C42*C6/(0.85*C5*(C7*1000)))/2)/1000000</f>
+        <v/>
+      </c>
+      <c r="D59" s="9" t="inlineStr">
+        <is>
+          <t>kN.m</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>Ve = (Mpr- + Mpr+)/Ln</t>
+        </is>
+      </c>
+      <c r="C60" s="9">
+        <f>(C58+C59)/C14</f>
+        <v/>
+      </c>
+      <c r="D60" s="9" t="inlineStr">
+        <is>
+          <t>kN</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>V de diseno = max(Vu, Ve)</t>
+        </is>
+      </c>
+      <c r="C61" s="14">
+        <f>MAX(C20,C60)</f>
+        <v/>
+      </c>
+      <c r="D61" s="9" t="inlineStr">
+        <is>
+          <t>kN</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>7. TORSION  (phi=0.75, theta=45)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>Acp = b h</t>
+        </is>
+      </c>
+      <c r="C64" s="9">
+        <f>(C7*1000)*(C8*1000)</f>
+        <v/>
+      </c>
+      <c r="D64" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+      <c r="J64" s="7" t="inlineStr">
+        <is>
+          <t>Estribo total = Av/s(cortante) + 2(At/s). Al se reparte en el perimetro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>pcp = 2(b+h)</t>
+        </is>
+      </c>
+      <c r="C65" s="9">
+        <f>2*((C7*1000)+(C8*1000))</f>
+        <v/>
+      </c>
+      <c r="D65" s="9" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>T umbral = phi 0.083 raiz(f'c) Acp2/pcp</t>
+        </is>
+      </c>
+      <c r="C66" s="9">
+        <f>0.75*0.083*SQRT(C5)*(C64^2/C65)/1000000</f>
+        <v/>
+      </c>
+      <c r="D66" s="9" t="inlineStr">
+        <is>
+          <t>kN.m</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>Requiere torsion?</t>
+        </is>
+      </c>
+      <c r="C67" s="14">
+        <f>IF(C21&gt;C66,"SI - disenar","No - despreciable")</f>
+        <v/>
+      </c>
+      <c r="D67" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>Aoh = (b-2r)(h-2r)</t>
+        </is>
+      </c>
+      <c r="C68" s="9">
+        <f>((C7*1000)-2*C9*1000)*((C8*1000)-2*C9*1000)</f>
+        <v/>
+      </c>
+      <c r="D68" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>ph = 2[(b-2r)+(h-2r)]</t>
+        </is>
+      </c>
+      <c r="C69" s="9">
+        <f>2*(((C7*1000)-2*C9*1000)+((C8*1000)-2*C9*1000))</f>
+        <v/>
+      </c>
+      <c r="D69" s="9" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>Ao = 0.85 Aoh</t>
+        </is>
+      </c>
+      <c r="C70" s="9">
+        <f>0.85*C68</f>
+        <v/>
+      </c>
+      <c r="D70" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>At/s (estribo torsion)</t>
+        </is>
+      </c>
+      <c r="C71" s="15">
+        <f>IF(C21&gt;C66,C21*1000000/(0.75*2*C70*C6),0)</f>
+        <v/>
+      </c>
+      <c r="D71" s="9" t="inlineStr">
+        <is>
+          <t>mm2/mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>Al (long. por torsion)</t>
+        </is>
+      </c>
+      <c r="C72" s="15">
+        <f>IF(C21&gt;C66,C71*C69,0)</f>
+        <v/>
+      </c>
+      <c r="D72" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>8. DEFLEXION (C.9.5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>h min = Ln/18.5</t>
+        </is>
+      </c>
+      <c r="C75" s="9">
+        <f>C14/18.5</f>
+        <v/>
+      </c>
+      <c r="D75" s="9" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>VERIFICACION</t>
+        </is>
+      </c>
+      <c r="C76" s="11">
+        <f>IF(C8&gt;=C75,"CUMPLE","REVISAR")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>9. DESPIECE (resumen)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="40" customHeight="1">
+      <c r="B79" s="7" t="inlineStr">
+        <is>
+          <t>Acero superior: As(-) corrido + bastones en zona negativa (Ln/4 + ld). Inferior: As(+) corrido. Estribos #3: confinamiento @ s_adoptar en 2h desde cada cara, resto @ d/2. Ganchos sismicos 135 grados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B79:J80"/>
+    <mergeCell ref="B2:J2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Agregar Cuadro de Viguetas por tipo de luz (entrepiso + cubierta), diseno completo viguetas/vigas/riostras por tipos
</commit_message>
<xml_diff>
--- a/Proyectos/Diseno-Estructural/Insumos/Diseno-Estructural-Calculos.xlsx
+++ b/Proyectos/Diseno-Estructural/Insumos/Diseno-Estructural-Calculos.xlsx
@@ -8,10 +8,11 @@
   </bookViews>
   <sheets>
     <sheet name="Irregularidades" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Cuadro Vigas-Riostras" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Diseno Vigas" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Diseno Riostras" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Diseno Viguetas" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Cuadro Viguetas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Cuadro Vigas-Riostras" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Diseno Vigas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Diseno Riostras" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Diseno Viguetas" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -182,7 +183,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -263,6 +264,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1780,6 +1784,800 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="B2:N29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="23" t="inlineStr">
+        <is>
+          <t>CUADRO DE VIGUETAS POR TIPO DE LUZ  (losa aligerada, viga T, gravedad)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Geometria y materiales (comunes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="27" t="inlineStr">
+        <is>
+          <t>f'c [MPa]</t>
+        </is>
+      </c>
+      <c r="C5" s="28" t="n">
+        <v>28</v>
+      </c>
+      <c r="D5" s="27" t="inlineStr">
+        <is>
+          <t>fy [MPa]</t>
+        </is>
+      </c>
+      <c r="E5" s="28" t="n">
+        <v>420</v>
+      </c>
+      <c r="F5" s="27" t="inlineStr">
+        <is>
+          <t>bw [m]</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H5" s="27" t="inlineStr">
+        <is>
+          <t>h [m]</t>
+        </is>
+      </c>
+      <c r="I5" s="28" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="J5" s="27" t="inlineStr">
+        <is>
+          <t>hf [m]</t>
+        </is>
+      </c>
+      <c r="K5" s="28" t="n">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="27" t="inlineStr">
+        <is>
+          <t>sv [m]</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D6" s="27" t="inlineStr">
+        <is>
+          <t>recubr [m]</t>
+        </is>
+      </c>
+      <c r="E6" s="28" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F6" s="27" t="inlineStr">
+        <is>
+          <t>Diam barra</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="H6" s="27" t="inlineStr">
+        <is>
+          <t>#4 Area</t>
+        </is>
+      </c>
+      <c r="I6" s="28" t="n">
+        <v>129</v>
+      </c>
+      <c r="J6" s="27" t="inlineStr">
+        <is>
+          <t>ancho apoyo [m]</t>
+        </is>
+      </c>
+      <c r="K6" s="28" t="n">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>d [mm]</t>
+        </is>
+      </c>
+      <c r="C7" s="34">
+        <f>I5*1000-E6*1000-G6/2</f>
+        <v/>
+      </c>
+      <c r="D7" s="24" t="inlineStr">
+        <is>
+          <t>As min [mm2]</t>
+        </is>
+      </c>
+      <c r="F7" s="34">
+        <f>MAX(0.25*SQRT(C5)/E5,1.4/E5)*G5*1000*C7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Vigueta continua: M- = wu Ln2/10 (apoyo), M+ = wu Ln2/14 (centro), Vu = 1.15 wu Ln/2.  Ln = L_ejes - ancho apoyo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>VIGUETAS DE ENTREPISO  (carga viva recreativa)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="27" t="inlineStr">
+        <is>
+          <t>wD [kN/m2]</t>
+        </is>
+      </c>
+      <c r="C11" s="28" t="n">
+        <v>7.04</v>
+      </c>
+      <c r="D11" s="27" t="inlineStr">
+        <is>
+          <t>wL [kN/m2]</t>
+        </is>
+      </c>
+      <c r="E11" s="28" t="n">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="29" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C12" s="29" t="inlineStr">
+        <is>
+          <t>L ejes [m]</t>
+        </is>
+      </c>
+      <c r="D12" s="29" t="inlineStr">
+        <is>
+          <t>Ln [m]</t>
+        </is>
+      </c>
+      <c r="E12" s="29" t="inlineStr">
+        <is>
+          <t>wu [kN/m]</t>
+        </is>
+      </c>
+      <c r="F12" s="29" t="inlineStr">
+        <is>
+          <t>M- [kN.m]</t>
+        </is>
+      </c>
+      <c r="G12" s="29" t="inlineStr">
+        <is>
+          <t>M+ [kN.m]</t>
+        </is>
+      </c>
+      <c r="H12" s="29" t="inlineStr">
+        <is>
+          <t>Vu [kN]</t>
+        </is>
+      </c>
+      <c r="I12" s="29" t="inlineStr">
+        <is>
+          <t>bf [mm]</t>
+        </is>
+      </c>
+      <c r="J12" s="29" t="inlineStr">
+        <is>
+          <t>As+ [mm2]</t>
+        </is>
+      </c>
+      <c r="K12" s="29" t="inlineStr">
+        <is>
+          <t>N #4+</t>
+        </is>
+      </c>
+      <c r="L12" s="29" t="inlineStr">
+        <is>
+          <t>As- [mm2]</t>
+        </is>
+      </c>
+      <c r="M12" s="29" t="inlineStr">
+        <is>
+          <t>N #4-</t>
+        </is>
+      </c>
+      <c r="N12" s="29" t="inlineStr">
+        <is>
+          <t>Estribos?</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="30" t="inlineStr">
+        <is>
+          <t>VT-1</t>
+        </is>
+      </c>
+      <c r="C13" s="28" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="D13" s="31">
+        <f>C13-$K$6</f>
+        <v/>
+      </c>
+      <c r="E13" s="31">
+        <f>(1.2*C11+1.6*E11)*$C$6</f>
+        <v/>
+      </c>
+      <c r="F13" s="31">
+        <f>E13*D13^2/10</f>
+        <v/>
+      </c>
+      <c r="G13" s="31">
+        <f>E13*D13^2/14</f>
+        <v/>
+      </c>
+      <c r="H13" s="31">
+        <f>1.15*E13*D13/2</f>
+        <v/>
+      </c>
+      <c r="I13" s="31">
+        <f>MIN(D13*1000/4,($G$5*1000)+16*$K$5*1000,$C$6*1000)</f>
+        <v/>
+      </c>
+      <c r="J13" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(G13*1000000/(0.9*I13*$C$7^2))/(0.85*$C$5)))*I13*$C$7,$F$7)</f>
+        <v/>
+      </c>
+      <c r="K13" s="33">
+        <f>ROUNDUP(J13/$I$6,0)</f>
+        <v/>
+      </c>
+      <c r="L13" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(F13*1000000/(0.9*($G$5*1000)*$C$7^2))/(0.85*$C$5)))*($G$5*1000)*$C$7,$F$7)</f>
+        <v/>
+      </c>
+      <c r="M13" s="33">
+        <f>ROUNDUP(L13/$I$6,0)</f>
+        <v/>
+      </c>
+      <c r="N13" s="31">
+        <f>IF(H13&lt;=0.75*1.1*(0.17*SQRT($C$5)*($G$5*1000)*$C$7/1000),"No","Si")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="30" t="inlineStr">
+        <is>
+          <t>VT-2</t>
+        </is>
+      </c>
+      <c r="C14" s="28" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="D14" s="31">
+        <f>C14-$K$6</f>
+        <v/>
+      </c>
+      <c r="E14" s="31">
+        <f>(1.2*C11+1.6*E11)*$C$6</f>
+        <v/>
+      </c>
+      <c r="F14" s="31">
+        <f>E14*D14^2/10</f>
+        <v/>
+      </c>
+      <c r="G14" s="31">
+        <f>E14*D14^2/14</f>
+        <v/>
+      </c>
+      <c r="H14" s="31">
+        <f>1.15*E14*D14/2</f>
+        <v/>
+      </c>
+      <c r="I14" s="31">
+        <f>MIN(D14*1000/4,($G$5*1000)+16*$K$5*1000,$C$6*1000)</f>
+        <v/>
+      </c>
+      <c r="J14" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(G14*1000000/(0.9*I14*$C$7^2))/(0.85*$C$5)))*I14*$C$7,$F$7)</f>
+        <v/>
+      </c>
+      <c r="K14" s="33">
+        <f>ROUNDUP(J14/$I$6,0)</f>
+        <v/>
+      </c>
+      <c r="L14" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(F14*1000000/(0.9*($G$5*1000)*$C$7^2))/(0.85*$C$5)))*($G$5*1000)*$C$7,$F$7)</f>
+        <v/>
+      </c>
+      <c r="M14" s="33">
+        <f>ROUNDUP(L14/$I$6,0)</f>
+        <v/>
+      </c>
+      <c r="N14" s="31">
+        <f>IF(H14&lt;=0.75*1.1*(0.17*SQRT($C$5)*($G$5*1000)*$C$7/1000),"No","Si")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="30" t="inlineStr">
+        <is>
+          <t>VT-3</t>
+        </is>
+      </c>
+      <c r="C15" s="28" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="D15" s="31">
+        <f>C15-$K$6</f>
+        <v/>
+      </c>
+      <c r="E15" s="31">
+        <f>(1.2*C11+1.6*E11)*$C$6</f>
+        <v/>
+      </c>
+      <c r="F15" s="31">
+        <f>E15*D15^2/10</f>
+        <v/>
+      </c>
+      <c r="G15" s="31">
+        <f>E15*D15^2/14</f>
+        <v/>
+      </c>
+      <c r="H15" s="31">
+        <f>1.15*E15*D15/2</f>
+        <v/>
+      </c>
+      <c r="I15" s="31">
+        <f>MIN(D15*1000/4,($G$5*1000)+16*$K$5*1000,$C$6*1000)</f>
+        <v/>
+      </c>
+      <c r="J15" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(G15*1000000/(0.9*I15*$C$7^2))/(0.85*$C$5)))*I15*$C$7,$F$7)</f>
+        <v/>
+      </c>
+      <c r="K15" s="33">
+        <f>ROUNDUP(J15/$I$6,0)</f>
+        <v/>
+      </c>
+      <c r="L15" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(F15*1000000/(0.9*($G$5*1000)*$C$7^2))/(0.85*$C$5)))*($G$5*1000)*$C$7,$F$7)</f>
+        <v/>
+      </c>
+      <c r="M15" s="33">
+        <f>ROUNDUP(L15/$I$6,0)</f>
+        <v/>
+      </c>
+      <c r="N15" s="31">
+        <f>IF(H15&lt;=0.75*1.1*(0.17*SQRT($C$5)*($G$5*1000)*$C$7/1000),"No","Si")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="30" t="inlineStr">
+        <is>
+          <t>VT-4</t>
+        </is>
+      </c>
+      <c r="C16" s="28" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="D16" s="31">
+        <f>C16-$K$6</f>
+        <v/>
+      </c>
+      <c r="E16" s="31">
+        <f>(1.2*C11+1.6*E11)*$C$6</f>
+        <v/>
+      </c>
+      <c r="F16" s="31">
+        <f>E16*D16^2/10</f>
+        <v/>
+      </c>
+      <c r="G16" s="31">
+        <f>E16*D16^2/14</f>
+        <v/>
+      </c>
+      <c r="H16" s="31">
+        <f>1.15*E16*D16/2</f>
+        <v/>
+      </c>
+      <c r="I16" s="31">
+        <f>MIN(D16*1000/4,($G$5*1000)+16*$K$5*1000,$C$6*1000)</f>
+        <v/>
+      </c>
+      <c r="J16" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(G16*1000000/(0.9*I16*$C$7^2))/(0.85*$C$5)))*I16*$C$7,$F$7)</f>
+        <v/>
+      </c>
+      <c r="K16" s="33">
+        <f>ROUNDUP(J16/$I$6,0)</f>
+        <v/>
+      </c>
+      <c r="L16" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(F16*1000000/(0.9*($G$5*1000)*$C$7^2))/(0.85*$C$5)))*($G$5*1000)*$C$7,$F$7)</f>
+        <v/>
+      </c>
+      <c r="M16" s="33">
+        <f>ROUNDUP(L16/$I$6,0)</f>
+        <v/>
+      </c>
+      <c r="N16" s="31">
+        <f>IF(H16&lt;=0.75*1.1*(0.17*SQRT($C$5)*($G$5*1000)*$C$7/1000),"No","Si")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>VIGUETAS DE CUBIERTA  (terraza social, L=5 kN/m2 - GOBIERNA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="27" t="inlineStr">
+        <is>
+          <t>wD [kN/m2]</t>
+        </is>
+      </c>
+      <c r="C19" s="28" t="n">
+        <v>4.376</v>
+      </c>
+      <c r="D19" s="27" t="inlineStr">
+        <is>
+          <t>wL [kN/m2]</t>
+        </is>
+      </c>
+      <c r="E19" s="28" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="29" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C20" s="29" t="inlineStr">
+        <is>
+          <t>L ejes [m]</t>
+        </is>
+      </c>
+      <c r="D20" s="29" t="inlineStr">
+        <is>
+          <t>Ln [m]</t>
+        </is>
+      </c>
+      <c r="E20" s="29" t="inlineStr">
+        <is>
+          <t>wu [kN/m]</t>
+        </is>
+      </c>
+      <c r="F20" s="29" t="inlineStr">
+        <is>
+          <t>M- [kN.m]</t>
+        </is>
+      </c>
+      <c r="G20" s="29" t="inlineStr">
+        <is>
+          <t>M+ [kN.m]</t>
+        </is>
+      </c>
+      <c r="H20" s="29" t="inlineStr">
+        <is>
+          <t>Vu [kN]</t>
+        </is>
+      </c>
+      <c r="I20" s="29" t="inlineStr">
+        <is>
+          <t>bf [mm]</t>
+        </is>
+      </c>
+      <c r="J20" s="29" t="inlineStr">
+        <is>
+          <t>As+ [mm2]</t>
+        </is>
+      </c>
+      <c r="K20" s="29" t="inlineStr">
+        <is>
+          <t>N #4+</t>
+        </is>
+      </c>
+      <c r="L20" s="29" t="inlineStr">
+        <is>
+          <t>As- [mm2]</t>
+        </is>
+      </c>
+      <c r="M20" s="29" t="inlineStr">
+        <is>
+          <t>N #4-</t>
+        </is>
+      </c>
+      <c r="N20" s="29" t="inlineStr">
+        <is>
+          <t>Estribos?</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="30" t="inlineStr">
+        <is>
+          <t>VT-1</t>
+        </is>
+      </c>
+      <c r="C21" s="28" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="D21" s="31">
+        <f>C21-$K$6</f>
+        <v/>
+      </c>
+      <c r="E21" s="31">
+        <f>(1.2*C19+1.6*E19)*$C$6</f>
+        <v/>
+      </c>
+      <c r="F21" s="31">
+        <f>E21*D21^2/10</f>
+        <v/>
+      </c>
+      <c r="G21" s="31">
+        <f>E21*D21^2/14</f>
+        <v/>
+      </c>
+      <c r="H21" s="31">
+        <f>1.15*E21*D21/2</f>
+        <v/>
+      </c>
+      <c r="I21" s="31">
+        <f>MIN(D21*1000/4,($G$5*1000)+16*$K$5*1000,$C$6*1000)</f>
+        <v/>
+      </c>
+      <c r="J21" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(G21*1000000/(0.9*I21*$C$7^2))/(0.85*$C$5)))*I21*$C$7,$F$7)</f>
+        <v/>
+      </c>
+      <c r="K21" s="33">
+        <f>ROUNDUP(J21/$I$6,0)</f>
+        <v/>
+      </c>
+      <c r="L21" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(F21*1000000/(0.9*($G$5*1000)*$C$7^2))/(0.85*$C$5)))*($G$5*1000)*$C$7,$F$7)</f>
+        <v/>
+      </c>
+      <c r="M21" s="33">
+        <f>ROUNDUP(L21/$I$6,0)</f>
+        <v/>
+      </c>
+      <c r="N21" s="31">
+        <f>IF(H21&lt;=0.75*1.1*(0.17*SQRT($C$5)*($G$5*1000)*$C$7/1000),"No","Si")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="30" t="inlineStr">
+        <is>
+          <t>VT-2</t>
+        </is>
+      </c>
+      <c r="C22" s="28" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="D22" s="31">
+        <f>C22-$K$6</f>
+        <v/>
+      </c>
+      <c r="E22" s="31">
+        <f>(1.2*C19+1.6*E19)*$C$6</f>
+        <v/>
+      </c>
+      <c r="F22" s="31">
+        <f>E22*D22^2/10</f>
+        <v/>
+      </c>
+      <c r="G22" s="31">
+        <f>E22*D22^2/14</f>
+        <v/>
+      </c>
+      <c r="H22" s="31">
+        <f>1.15*E22*D22/2</f>
+        <v/>
+      </c>
+      <c r="I22" s="31">
+        <f>MIN(D22*1000/4,($G$5*1000)+16*$K$5*1000,$C$6*1000)</f>
+        <v/>
+      </c>
+      <c r="J22" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(G22*1000000/(0.9*I22*$C$7^2))/(0.85*$C$5)))*I22*$C$7,$F$7)</f>
+        <v/>
+      </c>
+      <c r="K22" s="33">
+        <f>ROUNDUP(J22/$I$6,0)</f>
+        <v/>
+      </c>
+      <c r="L22" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(F22*1000000/(0.9*($G$5*1000)*$C$7^2))/(0.85*$C$5)))*($G$5*1000)*$C$7,$F$7)</f>
+        <v/>
+      </c>
+      <c r="M22" s="33">
+        <f>ROUNDUP(L22/$I$6,0)</f>
+        <v/>
+      </c>
+      <c r="N22" s="31">
+        <f>IF(H22&lt;=0.75*1.1*(0.17*SQRT($C$5)*($G$5*1000)*$C$7/1000),"No","Si")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="30" t="inlineStr">
+        <is>
+          <t>VT-3</t>
+        </is>
+      </c>
+      <c r="C23" s="28" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="D23" s="31">
+        <f>C23-$K$6</f>
+        <v/>
+      </c>
+      <c r="E23" s="31">
+        <f>(1.2*C19+1.6*E19)*$C$6</f>
+        <v/>
+      </c>
+      <c r="F23" s="31">
+        <f>E23*D23^2/10</f>
+        <v/>
+      </c>
+      <c r="G23" s="31">
+        <f>E23*D23^2/14</f>
+        <v/>
+      </c>
+      <c r="H23" s="31">
+        <f>1.15*E23*D23/2</f>
+        <v/>
+      </c>
+      <c r="I23" s="31">
+        <f>MIN(D23*1000/4,($G$5*1000)+16*$K$5*1000,$C$6*1000)</f>
+        <v/>
+      </c>
+      <c r="J23" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(G23*1000000/(0.9*I23*$C$7^2))/(0.85*$C$5)))*I23*$C$7,$F$7)</f>
+        <v/>
+      </c>
+      <c r="K23" s="33">
+        <f>ROUNDUP(J23/$I$6,0)</f>
+        <v/>
+      </c>
+      <c r="L23" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(F23*1000000/(0.9*($G$5*1000)*$C$7^2))/(0.85*$C$5)))*($G$5*1000)*$C$7,$F$7)</f>
+        <v/>
+      </c>
+      <c r="M23" s="33">
+        <f>ROUNDUP(L23/$I$6,0)</f>
+        <v/>
+      </c>
+      <c r="N23" s="31">
+        <f>IF(H23&lt;=0.75*1.1*(0.17*SQRT($C$5)*($G$5*1000)*$C$7/1000),"No","Si")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="30" t="inlineStr">
+        <is>
+          <t>VT-4</t>
+        </is>
+      </c>
+      <c r="C24" s="28" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="D24" s="31">
+        <f>C24-$K$6</f>
+        <v/>
+      </c>
+      <c r="E24" s="31">
+        <f>(1.2*C19+1.6*E19)*$C$6</f>
+        <v/>
+      </c>
+      <c r="F24" s="31">
+        <f>E24*D24^2/10</f>
+        <v/>
+      </c>
+      <c r="G24" s="31">
+        <f>E24*D24^2/14</f>
+        <v/>
+      </c>
+      <c r="H24" s="31">
+        <f>1.15*E24*D24/2</f>
+        <v/>
+      </c>
+      <c r="I24" s="31">
+        <f>MIN(D24*1000/4,($G$5*1000)+16*$K$5*1000,$C$6*1000)</f>
+        <v/>
+      </c>
+      <c r="J24" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(G24*1000000/(0.9*I24*$C$7^2))/(0.85*$C$5)))*I24*$C$7,$F$7)</f>
+        <v/>
+      </c>
+      <c r="K24" s="33">
+        <f>ROUNDUP(J24/$I$6,0)</f>
+        <v/>
+      </c>
+      <c r="L24" s="32">
+        <f>MAX((0.85*$C$5/$E$5)*(1-SQRT(1-2*(F24*1000000/(0.9*($G$5*1000)*$C$7^2))/(0.85*$C$5)))*($G$5*1000)*$C$7,$F$7)</f>
+        <v/>
+      </c>
+      <c r="M24" s="33">
+        <f>ROUNDUP(L24/$I$6,0)</f>
+        <v/>
+      </c>
+      <c r="N24" s="31">
+        <f>IF(H24&lt;=0.75*1.1*(0.17*SQRT($C$5)*($G$5*1000)*$C$7/1000),"No","Si")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>Despiece</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="46" customHeight="1">
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Todas las viguetas: refuerzo inferior As(+) corrido + refuerzo superior As(-) sobre apoyos (bastones Ln/4 + ld). Como las solicitaciones son bajas, casi todas requieren el As minimo (2 #4). Sin estribos (Vu &lt;= phi 1.1 Vc). Loseta con malla de retraccion Ø6 @ 250 mm (As=0.0018*b*hf). f'c=28 MPa, fy=420 MPa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28"/>
+    <row r="29"/>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B8:N8"/>
+    <mergeCell ref="B18:N18"/>
+    <mergeCell ref="B2:N2"/>
+    <mergeCell ref="B10:N10"/>
+    <mergeCell ref="B27:N29"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="B2:O25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1895,6 +2693,19 @@
           <t>VIGAS DE CARGA - VC 40x30</t>
         </is>
       </c>
+      <c r="C9" s="25" t="n"/>
+      <c r="D9" s="25" t="n"/>
+      <c r="E9" s="25" t="n"/>
+      <c r="F9" s="25" t="n"/>
+      <c r="G9" s="25" t="n"/>
+      <c r="H9" s="25" t="n"/>
+      <c r="I9" s="25" t="n"/>
+      <c r="J9" s="25" t="n"/>
+      <c r="K9" s="25" t="n"/>
+      <c r="L9" s="25" t="n"/>
+      <c r="M9" s="25" t="n"/>
+      <c r="N9" s="25" t="n"/>
+      <c r="O9" s="26" t="n"/>
     </row>
     <row r="10">
       <c r="B10" s="29" t="inlineStr">
@@ -2133,6 +2944,19 @@
           <t>RIOSTRAS / VIGAS DE RIGIDEZ - VR 40x35</t>
         </is>
       </c>
+      <c r="C15" s="25" t="n"/>
+      <c r="D15" s="25" t="n"/>
+      <c r="E15" s="25" t="n"/>
+      <c r="F15" s="25" t="n"/>
+      <c r="G15" s="25" t="n"/>
+      <c r="H15" s="25" t="n"/>
+      <c r="I15" s="25" t="n"/>
+      <c r="J15" s="25" t="n"/>
+      <c r="K15" s="25" t="n"/>
+      <c r="L15" s="25" t="n"/>
+      <c r="M15" s="25" t="n"/>
+      <c r="N15" s="25" t="n"/>
+      <c r="O15" s="26" t="n"/>
     </row>
     <row r="16">
       <c r="B16" s="29" t="inlineStr">
@@ -2442,1033 +3266,6 @@
     <mergeCell ref="B15:O15"/>
     <mergeCell ref="B7:O7"/>
     <mergeCell ref="B23:O25"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="B2:J80"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="46" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="2">
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>DISENO DE VIGAS DE CARGA  (VC 40x30) - NSR-10 / ACI 318 (DMO)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>1. DATOS Y GEOMETRIA</t>
-        </is>
-      </c>
-      <c r="J4" s="7" t="inlineStr">
-        <is>
-          <t>Celdas azules = entrada</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>f'c</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="n">
-        <v>28</v>
-      </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>MPa</t>
-        </is>
-      </c>
-      <c r="J5" s="7" t="inlineStr">
-        <is>
-          <t>phi=0.90 flexion - phi=0.75 cortante y torsion - rho_max(DMO)=0.025</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>fy = fyt</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="n">
-        <v>420</v>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>MPa</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>b (ancho)</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>h (alto)</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>recubrimiento r</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Diam estribo</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>mm #3</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Diam barra long.</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="n">
-        <v>15.9</v>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>mm #5</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Area barra long.</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="n">
-        <v>199</v>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Area 2 ramas Av</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="n">
-        <v>142</v>
-      </c>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Luz libre Ln</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>d = h - r - est - bl/2</t>
-        </is>
-      </c>
-      <c r="C15" s="14">
-        <f>C8*1000-C9*1000-C10-C11/2</f>
-        <v/>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>2. SOLICITACIONES (envolvente SAP, sismo / R=5)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Mu (-) negativo</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="n">
-        <v>142</v>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>kN.m</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Mu (+) positivo</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="n">
-        <v>101</v>
-      </c>
-      <c r="D19" s="9" t="inlineStr">
-        <is>
-          <t>kN.m</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>Vu cortante</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="n">
-        <v>108</v>
-      </c>
-      <c r="D20" s="9" t="inlineStr">
-        <is>
-          <t>kN</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Tu torsion</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="n">
-        <v>20</v>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
-        <is>
-          <t>kN.m</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>3. FLEXION - Momento NEGATIVO (acero superior)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>Rn = Mu/(phi b d2)</t>
-        </is>
-      </c>
-      <c r="C24" s="9">
-        <f>C18*1000000/(0.9*(C7*1000)*C15^2)</f>
-        <v/>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>MPa</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>rho requerido</t>
-        </is>
-      </c>
-      <c r="C25" s="9">
-        <f>(0.85*C5/C6)*(1-SQRT(1-2*C24/(0.85*C5)))</f>
-        <v/>
-      </c>
-      <c r="D25" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>As requerido</t>
-        </is>
-      </c>
-      <c r="C26" s="9">
-        <f>C25*(C7*1000)*C15</f>
-        <v/>
-      </c>
-      <c r="D26" s="9" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>As minimo (C.10.5)</t>
-        </is>
-      </c>
-      <c r="C27" s="9">
-        <f>MAX(0.25*SQRT(C5)/C6,1.4/C6)*(C7*1000)*C15</f>
-        <v/>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>As maximo (rho=0.025)</t>
-        </is>
-      </c>
-      <c r="C28" s="9">
-        <f>0.025*(C7*1000)*C15</f>
-        <v/>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>As de diseno</t>
-        </is>
-      </c>
-      <c r="C29" s="15">
-        <f>MAX(C26,C27)</f>
-        <v/>
-      </c>
-      <c r="D29" s="9" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>N barras</t>
-        </is>
-      </c>
-      <c r="C30" s="14">
-        <f>ROUNDUP(C29/C12,0)</f>
-        <v/>
-      </c>
-      <c r="D30" s="9" t="inlineStr">
-        <is>
-          <t>u</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>As colocado</t>
-        </is>
-      </c>
-      <c r="C31" s="15">
-        <f>C30*C12</f>
-        <v/>
-      </c>
-      <c r="D31" s="9" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>a (bloque comp.)</t>
-        </is>
-      </c>
-      <c r="C32" s="9">
-        <f>C31*C6/(0.85*C5*(C7*1000))</f>
-        <v/>
-      </c>
-      <c r="D32" s="9" t="inlineStr">
-        <is>
-          <t>mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>phiMn</t>
-        </is>
-      </c>
-      <c r="C33" s="14">
-        <f>0.9*C31*C6*(C15-C32/2)/1000000</f>
-        <v/>
-      </c>
-      <c r="D33" s="9" t="inlineStr">
-        <is>
-          <t>kN.m</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="6" t="inlineStr">
-        <is>
-          <t>VERIFICACION flexion (-)</t>
-        </is>
-      </c>
-      <c r="C34" s="11">
-        <f>IF(AND(C33&gt;=C18,C29&lt;=C28,C29&gt;=C27),"CUMPLE","REVISAR")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>4. FLEXION - Momento POSITIVO (acero inferior)</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>Rn</t>
-        </is>
-      </c>
-      <c r="C37" s="9">
-        <f>C19*1000000/(0.9*(C7*1000)*C15^2)</f>
-        <v/>
-      </c>
-      <c r="D37" s="9" t="inlineStr">
-        <is>
-          <t>MPa</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>rho requerido</t>
-        </is>
-      </c>
-      <c r="C38" s="9">
-        <f>(0.85*C5/C6)*(1-SQRT(1-2*C37/(0.85*C5)))</f>
-        <v/>
-      </c>
-      <c r="D38" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>As requerido</t>
-        </is>
-      </c>
-      <c r="C39" s="9">
-        <f>C38*(C7*1000)*C15</f>
-        <v/>
-      </c>
-      <c r="D39" s="9" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>As de diseno (&gt;= As min)</t>
-        </is>
-      </c>
-      <c r="C40" s="15">
-        <f>MAX(C39,C27)</f>
-        <v/>
-      </c>
-      <c r="D40" s="9" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>N barras</t>
-        </is>
-      </c>
-      <c r="C41" s="14">
-        <f>ROUNDUP(C40/C12,0)</f>
-        <v/>
-      </c>
-      <c r="D41" s="9" t="inlineStr">
-        <is>
-          <t>u</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>As colocado</t>
-        </is>
-      </c>
-      <c r="C42" s="15">
-        <f>C41*C12</f>
-        <v/>
-      </c>
-      <c r="D42" s="9" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="B43" s="4" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="C43" s="9">
-        <f>C42*C6/(0.85*C5*(C7*1000))</f>
-        <v/>
-      </c>
-      <c r="D43" s="9" t="inlineStr">
-        <is>
-          <t>mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="B44" s="4" t="inlineStr">
-        <is>
-          <t>phiMn</t>
-        </is>
-      </c>
-      <c r="C44" s="14">
-        <f>0.9*C42*C6*(C15-C43/2)/1000000</f>
-        <v/>
-      </c>
-      <c r="D44" s="9" t="inlineStr">
-        <is>
-          <t>kN.m</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="B45" s="6" t="inlineStr">
-        <is>
-          <t>VERIFICACION flexion (+)</t>
-        </is>
-      </c>
-      <c r="C45" s="11">
-        <f>IF(C44&gt;=C19,"CUMPLE","REVISAR")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>5. CORTANTE  (phi=0.75)</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="B48" s="4" t="inlineStr">
-        <is>
-          <t>Vc = 0.17 raiz(f'c) b d</t>
-        </is>
-      </c>
-      <c r="C48" s="9">
-        <f>0.17*SQRT(C5)*(C7*1000)*C15/1000</f>
-        <v/>
-      </c>
-      <c r="D48" s="9" t="inlineStr">
-        <is>
-          <t>kN</t>
-        </is>
-      </c>
-      <c r="J48" s="7" t="inlineStr">
-        <is>
-          <t>Estribos #3 de 2 ramas. Confinamiento = 2h desde cada cara del nudo (DMO C.21.3.4).</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="B49" s="4" t="inlineStr">
-        <is>
-          <t>phiVc</t>
-        </is>
-      </c>
-      <c r="C49" s="9">
-        <f>0.75*C48</f>
-        <v/>
-      </c>
-      <c r="D49" s="9" t="inlineStr">
-        <is>
-          <t>kN</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="B50" s="4" t="inlineStr">
-        <is>
-          <t>Vs requerido = Vu/phi - Vc</t>
-        </is>
-      </c>
-      <c r="C50" s="9">
-        <f>MAX(C20/0.75-C48,0)</f>
-        <v/>
-      </c>
-      <c r="D50" s="9" t="inlineStr">
-        <is>
-          <t>kN</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="B51" s="4" t="inlineStr">
-        <is>
-          <t>Vs max = 0.66 raiz(f'c) b d</t>
-        </is>
-      </c>
-      <c r="C51" s="9">
-        <f>0.66*SQRT(C5)*(C7*1000)*C15/1000</f>
-        <v/>
-      </c>
-      <c r="D51" s="9" t="inlineStr">
-        <is>
-          <t>kN</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="B52" s="4" t="inlineStr">
-        <is>
-          <t>s requerido = Av fyt d/Vs</t>
-        </is>
-      </c>
-      <c r="C52" s="9">
-        <f>IF(C50&gt;0,C13*C6*C15/(C50*1000),300)</f>
-        <v/>
-      </c>
-      <c r="D52" s="9" t="inlineStr">
-        <is>
-          <t>mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="B53" s="4" t="inlineStr">
-        <is>
-          <t>s max confinamiento DMO</t>
-        </is>
-      </c>
-      <c r="C53" s="9">
-        <f>MIN(C15/4,6*C11,150)</f>
-        <v/>
-      </c>
-      <c r="D53" s="9" t="inlineStr">
-        <is>
-          <t>mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="B54" s="4" t="inlineStr">
-        <is>
-          <t>Separacion a adoptar</t>
-        </is>
-      </c>
-      <c r="C54" s="14">
-        <f>IF(C50&gt;0,MIN(C52,C53),C53)</f>
-        <v/>
-      </c>
-      <c r="D54" s="9" t="inlineStr">
-        <is>
-          <t>mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="B55" s="6" t="inlineStr">
-        <is>
-          <t>VERIFICACION cortante</t>
-        </is>
-      </c>
-      <c r="C55" s="11">
-        <f>IF(C50&lt;=C51,"CUMPLE (seccion OK)","AUMENTAR SECCION")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57">
-      <c r="B57" s="2" t="inlineStr">
-        <is>
-          <t>6. CORTANTE POR CAPACIDAD (DMO C.21.3.4.2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="B58" s="4" t="inlineStr">
-        <is>
-          <t>Mpr(-) = 1.25 As fy (d-a/2)</t>
-        </is>
-      </c>
-      <c r="C58" s="9">
-        <f>1.25*C31*C6*(C15-(1.25*C31*C6/(0.85*C5*(C7*1000)))/2)/1000000</f>
-        <v/>
-      </c>
-      <c r="D58" s="9" t="inlineStr">
-        <is>
-          <t>kN.m</t>
-        </is>
-      </c>
-      <c r="J58" s="7" t="inlineStr">
-        <is>
-          <t>Sumar el cortante gravitacional del tramo a Ve. Gobierna el mayor entre Vu y Ve.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="B59" s="4" t="inlineStr">
-        <is>
-          <t>Mpr(+)</t>
-        </is>
-      </c>
-      <c r="C59" s="9">
-        <f>1.25*C42*C6*(C15-(1.25*C42*C6/(0.85*C5*(C7*1000)))/2)/1000000</f>
-        <v/>
-      </c>
-      <c r="D59" s="9" t="inlineStr">
-        <is>
-          <t>kN.m</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="B60" s="4" t="inlineStr">
-        <is>
-          <t>Ve = (Mpr- + Mpr+)/Ln</t>
-        </is>
-      </c>
-      <c r="C60" s="9">
-        <f>(C58+C59)/C14</f>
-        <v/>
-      </c>
-      <c r="D60" s="9" t="inlineStr">
-        <is>
-          <t>kN</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="B61" s="4" t="inlineStr">
-        <is>
-          <t>V de diseno = max(Vu, Ve)</t>
-        </is>
-      </c>
-      <c r="C61" s="14">
-        <f>MAX(C20,C60)</f>
-        <v/>
-      </c>
-      <c r="D61" s="9" t="inlineStr">
-        <is>
-          <t>kN</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="B63" s="2" t="inlineStr">
-        <is>
-          <t>7. TORSION  (phi=0.75, theta=45)</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="B64" s="4" t="inlineStr">
-        <is>
-          <t>Acp = b h</t>
-        </is>
-      </c>
-      <c r="C64" s="9">
-        <f>(C7*1000)*(C8*1000)</f>
-        <v/>
-      </c>
-      <c r="D64" s="9" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-      <c r="J64" s="7" t="inlineStr">
-        <is>
-          <t>Estribo total = Av/s(cortante) + 2(At/s). Al se reparte en el perimetro.</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="B65" s="4" t="inlineStr">
-        <is>
-          <t>pcp = 2(b+h)</t>
-        </is>
-      </c>
-      <c r="C65" s="9">
-        <f>2*((C7*1000)+(C8*1000))</f>
-        <v/>
-      </c>
-      <c r="D65" s="9" t="inlineStr">
-        <is>
-          <t>mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="B66" s="4" t="inlineStr">
-        <is>
-          <t>T umbral = phi 0.083 raiz(f'c) Acp2/pcp</t>
-        </is>
-      </c>
-      <c r="C66" s="9">
-        <f>0.75*0.083*SQRT(C5)*(C64^2/C65)/1000000</f>
-        <v/>
-      </c>
-      <c r="D66" s="9" t="inlineStr">
-        <is>
-          <t>kN.m</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="B67" s="4" t="inlineStr">
-        <is>
-          <t>Requiere torsion?</t>
-        </is>
-      </c>
-      <c r="C67" s="14">
-        <f>IF(C21&gt;C66,"SI - disenar","No - despreciable")</f>
-        <v/>
-      </c>
-      <c r="D67" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="B68" s="4" t="inlineStr">
-        <is>
-          <t>Aoh = (b-2r)(h-2r)</t>
-        </is>
-      </c>
-      <c r="C68" s="9">
-        <f>((C7*1000)-2*C9*1000)*((C8*1000)-2*C9*1000)</f>
-        <v/>
-      </c>
-      <c r="D68" s="9" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="B69" s="4" t="inlineStr">
-        <is>
-          <t>ph = 2[(b-2r)+(h-2r)]</t>
-        </is>
-      </c>
-      <c r="C69" s="9">
-        <f>2*(((C7*1000)-2*C9*1000)+((C8*1000)-2*C9*1000))</f>
-        <v/>
-      </c>
-      <c r="D69" s="9" t="inlineStr">
-        <is>
-          <t>mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="B70" s="4" t="inlineStr">
-        <is>
-          <t>Ao = 0.85 Aoh</t>
-        </is>
-      </c>
-      <c r="C70" s="9">
-        <f>0.85*C68</f>
-        <v/>
-      </c>
-      <c r="D70" s="9" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="B71" s="4" t="inlineStr">
-        <is>
-          <t>At/s (estribo torsion)</t>
-        </is>
-      </c>
-      <c r="C71" s="15">
-        <f>IF(C21&gt;C66,C21*1000000/(0.75*2*C70*C6),0)</f>
-        <v/>
-      </c>
-      <c r="D71" s="9" t="inlineStr">
-        <is>
-          <t>mm2/mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="B72" s="4" t="inlineStr">
-        <is>
-          <t>Al (long. por torsion)</t>
-        </is>
-      </c>
-      <c r="C72" s="15">
-        <f>IF(C21&gt;C66,C71*C69,0)</f>
-        <v/>
-      </c>
-      <c r="D72" s="9" t="inlineStr">
-        <is>
-          <t>mm2</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="B74" s="2" t="inlineStr">
-        <is>
-          <t>8. DEFLEXION (C.9.5)</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="B75" s="4" t="inlineStr">
-        <is>
-          <t>h min = Ln/18.5</t>
-        </is>
-      </c>
-      <c r="C75" s="9">
-        <f>C14/18.5</f>
-        <v/>
-      </c>
-      <c r="D75" s="9" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="B76" s="6" t="inlineStr">
-        <is>
-          <t>VERIFICACION</t>
-        </is>
-      </c>
-      <c r="C76" s="11">
-        <f>IF(C8&gt;=C75,"CUMPLE","REVISAR")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="78">
-      <c r="B78" s="2" t="inlineStr">
-        <is>
-          <t>9. DESPIECE (resumen)</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="40" customHeight="1">
-      <c r="B79" s="7" t="inlineStr">
-        <is>
-          <t>Acero superior: As(-) corrido + bastones en zona negativa (Ln/4 + ld). Inferior: As(+) corrido. Estribos #3: confinamiento @ s_adoptar en 2h desde cada cara, resto @ d/2. Ganchos sismicos 135 grados.</t>
-        </is>
-      </c>
-    </row>
-    <row r="80"/>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B79:J80"/>
-    <mergeCell ref="B2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3498,7 +3295,7 @@
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>DISENO DE RIOSTRAS / VIGAS DE RIGIDEZ  (VR 40x35) - NSR-10 / ACI 318 (DMO)</t>
+          <t>DISENO DE VIGAS DE CARGA  (VC 40x30) - NSR-10 / ACI 318 (DMO)</t>
         </is>
       </c>
     </row>
@@ -3556,7 +3353,7 @@
         </is>
       </c>
       <c r="C7" s="5" t="n">
-        <v>0.35</v>
+        <v>0.3</v>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
@@ -3661,7 +3458,7 @@
         </is>
       </c>
       <c r="C14" s="5" t="n">
-        <v>5.1</v>
+        <v>4.9</v>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
@@ -3699,7 +3496,7 @@
         </is>
       </c>
       <c r="C18" s="5" t="n">
-        <v>250</v>
+        <v>142</v>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
@@ -3714,7 +3511,7 @@
         </is>
       </c>
       <c r="C19" s="5" t="n">
-        <v>138</v>
+        <v>101</v>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
@@ -3729,7 +3526,7 @@
         </is>
       </c>
       <c r="C20" s="5" t="n">
-        <v>202</v>
+        <v>108</v>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
@@ -3744,7 +3541,7 @@
         </is>
       </c>
       <c r="C21" s="5" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
@@ -4502,6 +4299,1033 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:J80"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="46" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>DISENO DE RIOSTRAS / VIGAS DE RIGIDEZ  (VR 40x35) - NSR-10 / ACI 318 (DMO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>1. DATOS Y GEOMETRIA</t>
+        </is>
+      </c>
+      <c r="J4" s="7" t="inlineStr">
+        <is>
+          <t>Celdas azules = entrada</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>f'c</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>phi=0.90 flexion - phi=0.75 cortante y torsion - rho_max(DMO)=0.025</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>fy = fyt</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>420</v>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>b (ancho)</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>h (alto)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>recubrimiento r</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Diam estribo</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>mm #3</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Diam barra long.</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>mm #5</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Area barra long.</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>199</v>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Area 2 ramas Av</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>142</v>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Luz libre Ln</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>d = h - r - est - bl/2</t>
+        </is>
+      </c>
+      <c r="C15" s="14">
+        <f>C8*1000-C9*1000-C10-C11/2</f>
+        <v/>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>2. SOLICITACIONES (envolvente SAP, sismo / R=5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Mu (-) negativo</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>250</v>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>kN.m</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Mu (+) positivo</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>138</v>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>kN.m</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Vu cortante</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>202</v>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>kN</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Tu torsion</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>kN.m</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>3. FLEXION - Momento NEGATIVO (acero superior)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Rn = Mu/(phi b d2)</t>
+        </is>
+      </c>
+      <c r="C24" s="9">
+        <f>C18*1000000/(0.9*(C7*1000)*C15^2)</f>
+        <v/>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>rho requerido</t>
+        </is>
+      </c>
+      <c r="C25" s="9">
+        <f>(0.85*C5/C6)*(1-SQRT(1-2*C24/(0.85*C5)))</f>
+        <v/>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>As requerido</t>
+        </is>
+      </c>
+      <c r="C26" s="9">
+        <f>C25*(C7*1000)*C15</f>
+        <v/>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>As minimo (C.10.5)</t>
+        </is>
+      </c>
+      <c r="C27" s="9">
+        <f>MAX(0.25*SQRT(C5)/C6,1.4/C6)*(C7*1000)*C15</f>
+        <v/>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>As maximo (rho=0.025)</t>
+        </is>
+      </c>
+      <c r="C28" s="9">
+        <f>0.025*(C7*1000)*C15</f>
+        <v/>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>As de diseno</t>
+        </is>
+      </c>
+      <c r="C29" s="15">
+        <f>MAX(C26,C27)</f>
+        <v/>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>N barras</t>
+        </is>
+      </c>
+      <c r="C30" s="14">
+        <f>ROUNDUP(C29/C12,0)</f>
+        <v/>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>u</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>As colocado</t>
+        </is>
+      </c>
+      <c r="C31" s="15">
+        <f>C30*C12</f>
+        <v/>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>a (bloque comp.)</t>
+        </is>
+      </c>
+      <c r="C32" s="9">
+        <f>C31*C6/(0.85*C5*(C7*1000))</f>
+        <v/>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>phiMn</t>
+        </is>
+      </c>
+      <c r="C33" s="14">
+        <f>0.9*C31*C6*(C15-C32/2)/1000000</f>
+        <v/>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>kN.m</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>VERIFICACION flexion (-)</t>
+        </is>
+      </c>
+      <c r="C34" s="11">
+        <f>IF(AND(C33&gt;=C18,C29&lt;=C28,C29&gt;=C27),"CUMPLE","REVISAR")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>4. FLEXION - Momento POSITIVO (acero inferior)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Rn</t>
+        </is>
+      </c>
+      <c r="C37" s="9">
+        <f>C19*1000000/(0.9*(C7*1000)*C15^2)</f>
+        <v/>
+      </c>
+      <c r="D37" s="9" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>rho requerido</t>
+        </is>
+      </c>
+      <c r="C38" s="9">
+        <f>(0.85*C5/C6)*(1-SQRT(1-2*C37/(0.85*C5)))</f>
+        <v/>
+      </c>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>As requerido</t>
+        </is>
+      </c>
+      <c r="C39" s="9">
+        <f>C38*(C7*1000)*C15</f>
+        <v/>
+      </c>
+      <c r="D39" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>As de diseno (&gt;= As min)</t>
+        </is>
+      </c>
+      <c r="C40" s="15">
+        <f>MAX(C39,C27)</f>
+        <v/>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>N barras</t>
+        </is>
+      </c>
+      <c r="C41" s="14">
+        <f>ROUNDUP(C40/C12,0)</f>
+        <v/>
+      </c>
+      <c r="D41" s="9" t="inlineStr">
+        <is>
+          <t>u</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>As colocado</t>
+        </is>
+      </c>
+      <c r="C42" s="15">
+        <f>C41*C12</f>
+        <v/>
+      </c>
+      <c r="D42" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="C43" s="9">
+        <f>C42*C6/(0.85*C5*(C7*1000))</f>
+        <v/>
+      </c>
+      <c r="D43" s="9" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>phiMn</t>
+        </is>
+      </c>
+      <c r="C44" s="14">
+        <f>0.9*C42*C6*(C15-C43/2)/1000000</f>
+        <v/>
+      </c>
+      <c r="D44" s="9" t="inlineStr">
+        <is>
+          <t>kN.m</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>VERIFICACION flexion (+)</t>
+        </is>
+      </c>
+      <c r="C45" s="11">
+        <f>IF(C44&gt;=C19,"CUMPLE","REVISAR")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>5. CORTANTE  (phi=0.75)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Vc = 0.17 raiz(f'c) b d</t>
+        </is>
+      </c>
+      <c r="C48" s="9">
+        <f>0.17*SQRT(C5)*(C7*1000)*C15/1000</f>
+        <v/>
+      </c>
+      <c r="D48" s="9" t="inlineStr">
+        <is>
+          <t>kN</t>
+        </is>
+      </c>
+      <c r="J48" s="7" t="inlineStr">
+        <is>
+          <t>Estribos #3 de 2 ramas. Confinamiento = 2h desde cada cara del nudo (DMO C.21.3.4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>phiVc</t>
+        </is>
+      </c>
+      <c r="C49" s="9">
+        <f>0.75*C48</f>
+        <v/>
+      </c>
+      <c r="D49" s="9" t="inlineStr">
+        <is>
+          <t>kN</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Vs requerido = Vu/phi - Vc</t>
+        </is>
+      </c>
+      <c r="C50" s="9">
+        <f>MAX(C20/0.75-C48,0)</f>
+        <v/>
+      </c>
+      <c r="D50" s="9" t="inlineStr">
+        <is>
+          <t>kN</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Vs max = 0.66 raiz(f'c) b d</t>
+        </is>
+      </c>
+      <c r="C51" s="9">
+        <f>0.66*SQRT(C5)*(C7*1000)*C15/1000</f>
+        <v/>
+      </c>
+      <c r="D51" s="9" t="inlineStr">
+        <is>
+          <t>kN</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>s requerido = Av fyt d/Vs</t>
+        </is>
+      </c>
+      <c r="C52" s="9">
+        <f>IF(C50&gt;0,C13*C6*C15/(C50*1000),300)</f>
+        <v/>
+      </c>
+      <c r="D52" s="9" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>s max confinamiento DMO</t>
+        </is>
+      </c>
+      <c r="C53" s="9">
+        <f>MIN(C15/4,6*C11,150)</f>
+        <v/>
+      </c>
+      <c r="D53" s="9" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>Separacion a adoptar</t>
+        </is>
+      </c>
+      <c r="C54" s="14">
+        <f>IF(C50&gt;0,MIN(C52,C53),C53)</f>
+        <v/>
+      </c>
+      <c r="D54" s="9" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>VERIFICACION cortante</t>
+        </is>
+      </c>
+      <c r="C55" s="11">
+        <f>IF(C50&lt;=C51,"CUMPLE (seccion OK)","AUMENTAR SECCION")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>6. CORTANTE POR CAPACIDAD (DMO C.21.3.4.2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>Mpr(-) = 1.25 As fy (d-a/2)</t>
+        </is>
+      </c>
+      <c r="C58" s="9">
+        <f>1.25*C31*C6*(C15-(1.25*C31*C6/(0.85*C5*(C7*1000)))/2)/1000000</f>
+        <v/>
+      </c>
+      <c r="D58" s="9" t="inlineStr">
+        <is>
+          <t>kN.m</t>
+        </is>
+      </c>
+      <c r="J58" s="7" t="inlineStr">
+        <is>
+          <t>Sumar el cortante gravitacional del tramo a Ve. Gobierna el mayor entre Vu y Ve.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>Mpr(+)</t>
+        </is>
+      </c>
+      <c r="C59" s="9">
+        <f>1.25*C42*C6*(C15-(1.25*C42*C6/(0.85*C5*(C7*1000)))/2)/1000000</f>
+        <v/>
+      </c>
+      <c r="D59" s="9" t="inlineStr">
+        <is>
+          <t>kN.m</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>Ve = (Mpr- + Mpr+)/Ln</t>
+        </is>
+      </c>
+      <c r="C60" s="9">
+        <f>(C58+C59)/C14</f>
+        <v/>
+      </c>
+      <c r="D60" s="9" t="inlineStr">
+        <is>
+          <t>kN</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>V de diseno = max(Vu, Ve)</t>
+        </is>
+      </c>
+      <c r="C61" s="14">
+        <f>MAX(C20,C60)</f>
+        <v/>
+      </c>
+      <c r="D61" s="9" t="inlineStr">
+        <is>
+          <t>kN</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>7. TORSION  (phi=0.75, theta=45)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>Acp = b h</t>
+        </is>
+      </c>
+      <c r="C64" s="9">
+        <f>(C7*1000)*(C8*1000)</f>
+        <v/>
+      </c>
+      <c r="D64" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+      <c r="J64" s="7" t="inlineStr">
+        <is>
+          <t>Estribo total = Av/s(cortante) + 2(At/s). Al se reparte en el perimetro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>pcp = 2(b+h)</t>
+        </is>
+      </c>
+      <c r="C65" s="9">
+        <f>2*((C7*1000)+(C8*1000))</f>
+        <v/>
+      </c>
+      <c r="D65" s="9" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>T umbral = phi 0.083 raiz(f'c) Acp2/pcp</t>
+        </is>
+      </c>
+      <c r="C66" s="9">
+        <f>0.75*0.083*SQRT(C5)*(C64^2/C65)/1000000</f>
+        <v/>
+      </c>
+      <c r="D66" s="9" t="inlineStr">
+        <is>
+          <t>kN.m</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>Requiere torsion?</t>
+        </is>
+      </c>
+      <c r="C67" s="14">
+        <f>IF(C21&gt;C66,"SI - disenar","No - despreciable")</f>
+        <v/>
+      </c>
+      <c r="D67" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>Aoh = (b-2r)(h-2r)</t>
+        </is>
+      </c>
+      <c r="C68" s="9">
+        <f>((C7*1000)-2*C9*1000)*((C8*1000)-2*C9*1000)</f>
+        <v/>
+      </c>
+      <c r="D68" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>ph = 2[(b-2r)+(h-2r)]</t>
+        </is>
+      </c>
+      <c r="C69" s="9">
+        <f>2*(((C7*1000)-2*C9*1000)+((C8*1000)-2*C9*1000))</f>
+        <v/>
+      </c>
+      <c r="D69" s="9" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>Ao = 0.85 Aoh</t>
+        </is>
+      </c>
+      <c r="C70" s="9">
+        <f>0.85*C68</f>
+        <v/>
+      </c>
+      <c r="D70" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>At/s (estribo torsion)</t>
+        </is>
+      </c>
+      <c r="C71" s="15">
+        <f>IF(C21&gt;C66,C21*1000000/(0.75*2*C70*C6),0)</f>
+        <v/>
+      </c>
+      <c r="D71" s="9" t="inlineStr">
+        <is>
+          <t>mm2/mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>Al (long. por torsion)</t>
+        </is>
+      </c>
+      <c r="C72" s="15">
+        <f>IF(C21&gt;C66,C71*C69,0)</f>
+        <v/>
+      </c>
+      <c r="D72" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>8. DEFLEXION (C.9.5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>h min = Ln/18.5</t>
+        </is>
+      </c>
+      <c r="C75" s="9">
+        <f>C14/18.5</f>
+        <v/>
+      </c>
+      <c r="D75" s="9" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>VERIFICACION</t>
+        </is>
+      </c>
+      <c r="C76" s="11">
+        <f>IF(C8&gt;=C75,"CUMPLE","REVISAR")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>9. DESPIECE (resumen)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="40" customHeight="1">
+      <c r="B79" s="7" t="inlineStr">
+        <is>
+          <t>Acero superior: As(-) corrido + bastones en zona negativa (Ln/4 + ld). Inferior: As(+) corrido. Estribos #3: confinamiento @ s_adoptar en 2h desde cada cara, resto @ d/2. Ganchos sismicos 135 grados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B79:J80"/>
+    <mergeCell ref="B2:J2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Agregar calculo de longitud de gancho (ldh), longitud de cada barra (Ln+2ldh) y separacion de estribos (d/4 conf, d/2 centro) en Excel y memoria, segun guia del grupo
</commit_message>
<xml_diff>
--- a/Proyectos/Diseno-Estructural/Insumos/Diseno-Estructural-Calculos.xlsx
+++ b/Proyectos/Diseno-Estructural/Insumos/Diseno-Estructural-Calculos.xlsx
@@ -1,18 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Irregularidades" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Cuadro Viguetas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Cuadro Vigas-Riostras" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Diseno Vigas" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Diseno Riostras" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Diseno Viguetas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Irregularidades" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro Viguetas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro Vigas-Riostras" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diseno Vigas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diseno Riostras" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diseno Viguetas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Despiece y Longitudes" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -183,7 +184,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -267,6 +268,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1934,6 +1938,18 @@
           <t>VIGUETAS DE ENTREPISO  (carga viva recreativa)</t>
         </is>
       </c>
+      <c r="C10" s="25" t="n"/>
+      <c r="D10" s="25" t="n"/>
+      <c r="E10" s="25" t="n"/>
+      <c r="F10" s="25" t="n"/>
+      <c r="G10" s="25" t="n"/>
+      <c r="H10" s="25" t="n"/>
+      <c r="I10" s="25" t="n"/>
+      <c r="J10" s="25" t="n"/>
+      <c r="K10" s="25" t="n"/>
+      <c r="L10" s="25" t="n"/>
+      <c r="M10" s="25" t="n"/>
+      <c r="N10" s="26" t="n"/>
     </row>
     <row r="11">
       <c r="B11" s="27" t="inlineStr">
@@ -2242,6 +2258,18 @@
           <t>VIGUETAS DE CUBIERTA  (terraza social, L=5 kN/m2 - GOBIERNA)</t>
         </is>
       </c>
+      <c r="C18" s="25" t="n"/>
+      <c r="D18" s="25" t="n"/>
+      <c r="E18" s="25" t="n"/>
+      <c r="F18" s="25" t="n"/>
+      <c r="G18" s="25" t="n"/>
+      <c r="H18" s="25" t="n"/>
+      <c r="I18" s="25" t="n"/>
+      <c r="J18" s="25" t="n"/>
+      <c r="K18" s="25" t="n"/>
+      <c r="L18" s="25" t="n"/>
+      <c r="M18" s="25" t="n"/>
+      <c r="N18" s="26" t="n"/>
     </row>
     <row r="19">
       <c r="B19" s="27" t="inlineStr">
@@ -6003,4 +6031,495 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:I28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="23" t="inlineStr">
+        <is>
+          <t>DESPIECE: LONGITUDES DE DESARROLLO, GANCHOS Y ESTRIBOS  (NSR-10 C.7 y C.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>1. Parametros</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="27" t="inlineStr">
+        <is>
+          <t>f'c [MPa]</t>
+        </is>
+      </c>
+      <c r="C5" s="35" t="n">
+        <v>28</v>
+      </c>
+      <c r="D5" s="27" t="inlineStr">
+        <is>
+          <t>fy [MPa]</t>
+        </is>
+      </c>
+      <c r="E5" s="35" t="n">
+        <v>420</v>
+      </c>
+      <c r="F5" s="27" t="inlineStr">
+        <is>
+          <t>recubrimiento [mm]</t>
+        </is>
+      </c>
+      <c r="G5" s="35" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>ldh = 0.24 (fy/raiz f'c) db  (minimo 8db y 150 mm).  ld recto: C.12.2 (caso favorable).  Gancho 90: extension 12db.  Gancho 135 (estribo): extension 6db &gt;= 75 mm.  Diametro de doblado: 6db.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>2. Longitudes por diametro de barra [mm]</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="29" t="inlineStr">
+        <is>
+          <t>Barra</t>
+        </is>
+      </c>
+      <c r="C9" s="29" t="inlineStr">
+        <is>
+          <t>db</t>
+        </is>
+      </c>
+      <c r="D9" s="29" t="inlineStr">
+        <is>
+          <t>ld recto inf.</t>
+        </is>
+      </c>
+      <c r="E9" s="29" t="inlineStr">
+        <is>
+          <t>ld recto sup.</t>
+        </is>
+      </c>
+      <c r="F9" s="29" t="inlineStr">
+        <is>
+          <t>ldh (gancho)</t>
+        </is>
+      </c>
+      <c r="G9" s="29" t="inlineStr">
+        <is>
+          <t>Gancho 90 (12db)</t>
+        </is>
+      </c>
+      <c r="H9" s="29" t="inlineStr">
+        <is>
+          <t>Gancho 135 estribo</t>
+        </is>
+      </c>
+      <c r="I9" s="29" t="inlineStr">
+        <is>
+          <t>Diam. doblado (6db)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="30" t="inlineStr">
+        <is>
+          <t>Nº 3</t>
+        </is>
+      </c>
+      <c r="C10" s="35" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="D10" s="31">
+        <f>($E$5*1.0*0.8)/(1.1*SQRT($C$5)*2.5)*C10</f>
+        <v/>
+      </c>
+      <c r="E10" s="31">
+        <f>($E$5*1.3*0.8)/(1.1*SQRT($C$5)*2.5)*C10</f>
+        <v/>
+      </c>
+      <c r="F10" s="34">
+        <f>MAX(0.24*$E$5/SQRT($C$5)*C10,8*C10,150)</f>
+        <v/>
+      </c>
+      <c r="G10" s="31">
+        <f>12*C10</f>
+        <v/>
+      </c>
+      <c r="H10" s="31">
+        <f>MAX(6*C10,75)</f>
+        <v/>
+      </c>
+      <c r="I10" s="31">
+        <f>6*C10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="30" t="inlineStr">
+        <is>
+          <t>Nº 4</t>
+        </is>
+      </c>
+      <c r="C11" s="35" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="D11" s="31">
+        <f>($E$5*1.0*0.8)/(1.1*SQRT($C$5)*2.5)*C11</f>
+        <v/>
+      </c>
+      <c r="E11" s="31">
+        <f>($E$5*1.3*0.8)/(1.1*SQRT($C$5)*2.5)*C11</f>
+        <v/>
+      </c>
+      <c r="F11" s="34">
+        <f>MAX(0.24*$E$5/SQRT($C$5)*C11,8*C11,150)</f>
+        <v/>
+      </c>
+      <c r="G11" s="31">
+        <f>12*C11</f>
+        <v/>
+      </c>
+      <c r="H11" s="31">
+        <f>MAX(6*C11,75)</f>
+        <v/>
+      </c>
+      <c r="I11" s="31">
+        <f>6*C11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="30" t="inlineStr">
+        <is>
+          <t>Nº 5</t>
+        </is>
+      </c>
+      <c r="C12" s="35" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="D12" s="31">
+        <f>($E$5*1.0*0.8)/(1.1*SQRT($C$5)*2.5)*C12</f>
+        <v/>
+      </c>
+      <c r="E12" s="31">
+        <f>($E$5*1.3*0.8)/(1.1*SQRT($C$5)*2.5)*C12</f>
+        <v/>
+      </c>
+      <c r="F12" s="34">
+        <f>MAX(0.24*$E$5/SQRT($C$5)*C12,8*C12,150)</f>
+        <v/>
+      </c>
+      <c r="G12" s="31">
+        <f>12*C12</f>
+        <v/>
+      </c>
+      <c r="H12" s="31">
+        <f>MAX(6*C12,75)</f>
+        <v/>
+      </c>
+      <c r="I12" s="31">
+        <f>6*C12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>3. Longitud de corte de cada barra:  Ln + 2 ldh</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="29" t="inlineStr">
+        <is>
+          <t>Elemento</t>
+        </is>
+      </c>
+      <c r="C15" s="29" t="inlineStr">
+        <is>
+          <t>Barra</t>
+        </is>
+      </c>
+      <c r="D15" s="29" t="inlineStr">
+        <is>
+          <t>Luz libre Ln [m]</t>
+        </is>
+      </c>
+      <c r="E15" s="29" t="inlineStr">
+        <is>
+          <t>ldh [mm]</t>
+        </is>
+      </c>
+      <c r="F15" s="29" t="inlineStr">
+        <is>
+          <t>Longitud de barra [m]</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="31" t="inlineStr">
+        <is>
+          <t>Viga de carga VC</t>
+        </is>
+      </c>
+      <c r="C16" s="31" t="inlineStr">
+        <is>
+          <t>Nº 5</t>
+        </is>
+      </c>
+      <c r="D16" s="35" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="E16" s="31">
+        <f>F12</f>
+        <v/>
+      </c>
+      <c r="F16" s="34">
+        <f>(D16*1000+2*E16)/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="31" t="inlineStr">
+        <is>
+          <t>Riostra VR</t>
+        </is>
+      </c>
+      <c r="C17" s="31" t="inlineStr">
+        <is>
+          <t>Nº 5</t>
+        </is>
+      </c>
+      <c r="D17" s="35" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="E17" s="31">
+        <f>F12</f>
+        <v/>
+      </c>
+      <c r="F17" s="34">
+        <f>(D17*1000+2*E17)/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="31" t="inlineStr">
+        <is>
+          <t>Vigueta</t>
+        </is>
+      </c>
+      <c r="C18" s="31" t="inlineStr">
+        <is>
+          <t>Nº 4</t>
+        </is>
+      </c>
+      <c r="D18" s="35" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="E18" s="31">
+        <f>F11</f>
+        <v/>
+      </c>
+      <c r="F18" s="34">
+        <f>(D18*1000+2*E18)/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>La longitud incluye un gancho estandar a 90 grados en cada extremo, anclado dentro de las columnas. Para las barras superiores que no se cortan, el baston negativo se extiende Ln/4 mas la longitud de desarrollo desde la cara del apoyo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>4. Estribos (Nº 3) y zonas de confinamiento (DMO C.21.3.4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="29" t="inlineStr">
+        <is>
+          <t>Elemento</t>
+        </is>
+      </c>
+      <c r="C23" s="29" t="inlineStr">
+        <is>
+          <t>b [mm]</t>
+        </is>
+      </c>
+      <c r="D23" s="29" t="inlineStr">
+        <is>
+          <t>h [mm]</t>
+        </is>
+      </c>
+      <c r="E23" s="29" t="inlineStr">
+        <is>
+          <t>d [mm]</t>
+        </is>
+      </c>
+      <c r="F23" s="29" t="inlineStr">
+        <is>
+          <t>Zona confin. 2h [mm]</t>
+        </is>
+      </c>
+      <c r="G23" s="29" t="inlineStr">
+        <is>
+          <t>s confin. (d/4) [mm]</t>
+        </is>
+      </c>
+      <c r="H23" s="29" t="inlineStr">
+        <is>
+          <t>s centro (d/2) [mm]</t>
+        </is>
+      </c>
+      <c r="I23" s="29" t="inlineStr">
+        <is>
+          <t>Long. estribo [mm]</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="31" t="inlineStr">
+        <is>
+          <t>Viga de carga VC</t>
+        </is>
+      </c>
+      <c r="C24" s="35" t="n">
+        <v>300</v>
+      </c>
+      <c r="D24" s="35" t="n">
+        <v>400</v>
+      </c>
+      <c r="E24" s="35" t="n">
+        <v>342.6</v>
+      </c>
+      <c r="F24" s="31">
+        <f>2*D24</f>
+        <v/>
+      </c>
+      <c r="G24" s="34">
+        <f>MIN(E24/4,6*15.9,150)</f>
+        <v/>
+      </c>
+      <c r="H24" s="34">
+        <f>E24/2</f>
+        <v/>
+      </c>
+      <c r="I24" s="31">
+        <f>2*((C24-2*$G$5)+(D24-2*$G$5))+2*MAX(10*9.5,75)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="31" t="inlineStr">
+        <is>
+          <t>Riostra VR</t>
+        </is>
+      </c>
+      <c r="C25" s="35" t="n">
+        <v>350</v>
+      </c>
+      <c r="D25" s="35" t="n">
+        <v>400</v>
+      </c>
+      <c r="E25" s="35" t="n">
+        <v>342.6</v>
+      </c>
+      <c r="F25" s="31">
+        <f>2*D25</f>
+        <v/>
+      </c>
+      <c r="G25" s="34">
+        <f>MIN(E25/4,6*15.9,150)</f>
+        <v/>
+      </c>
+      <c r="H25" s="34">
+        <f>E25/2</f>
+        <v/>
+      </c>
+      <c r="I25" s="31">
+        <f>2*((C25-2*$G$5)+(D25-2*$G$5))+2*MAX(10*9.5,75)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="31" t="inlineStr">
+        <is>
+          <t>Vigueta</t>
+        </is>
+      </c>
+      <c r="C26" s="35" t="n">
+        <v>150</v>
+      </c>
+      <c r="D26" s="35" t="n">
+        <v>340</v>
+      </c>
+      <c r="E26" s="35" t="n">
+        <v>304</v>
+      </c>
+      <c r="F26" s="31">
+        <f>2*D26</f>
+        <v/>
+      </c>
+      <c r="G26" s="34">
+        <f>MIN(E26/4,6*15.9,150)</f>
+        <v/>
+      </c>
+      <c r="H26" s="34">
+        <f>E26/2</f>
+        <v/>
+      </c>
+      <c r="I26" s="31">
+        <f>2*((C26-2*$G$5)+(D26-2*$G$5))+2*MAX(10*9.5,75)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="28" customHeight="1">
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Estribos Nº 3 de dos ramas, con ganchos sismicos a 135 grados. En la zona de confinamiento (2h desde la cara de cada apoyo) se separan d/4; en el resto, d/2. La longitud del estribo incluye el perimetro interior mas los dos ganchos a 135 grados.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B28:I28"/>
+    <mergeCell ref="B6:I6"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B20:I20"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Corregir longitud de barras al metodo del grupo: superior Ln/4+ldh, inferior Ln+2ldh (segun entrega parcial de despiece)
</commit_message>
<xml_diff>
--- a/Proyectos/Diseno-Estructural/Insumos/Diseno-Estructural-Calculos.xlsx
+++ b/Proyectos/Diseno-Estructural/Insumos/Diseno-Estructural-Calculos.xlsx
@@ -184,7 +184,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -271,6 +271,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -6254,111 +6260,166 @@
     <row r="14">
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>3. Longitud de corte de cada barra:  Ln + 2 ldh</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="29" t="inlineStr">
-        <is>
-          <t>Elemento</t>
-        </is>
-      </c>
-      <c r="C15" s="29" t="inlineStr">
+          <t>3. Longitud de corte de cada barra</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="B15" s="36" t="inlineStr">
+        <is>
+          <t>Barras SUPERIORES (negativo, apoyos): L = Ln/4 + ldh.   Barras INFERIORES (positivo, centro): L = Ln + 2 ldh.   (metodo del grupo, NSR-10 C.12).</t>
+        </is>
+      </c>
+      <c r="C15" s="25" t="n"/>
+      <c r="D15" s="25" t="n"/>
+      <c r="E15" s="25" t="n"/>
+      <c r="F15" s="25" t="n"/>
+      <c r="G15" s="25" t="n"/>
+      <c r="H15" s="25" t="n"/>
+      <c r="I15" s="26" t="n"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="29" t="inlineStr">
+        <is>
+          <t>Posicion</t>
+        </is>
+      </c>
+      <c r="C16" s="29" t="inlineStr">
         <is>
           <t>Barra</t>
         </is>
       </c>
-      <c r="D15" s="29" t="inlineStr">
+      <c r="D16" s="29" t="inlineStr">
         <is>
           <t>Luz libre Ln [m]</t>
         </is>
       </c>
-      <c r="E15" s="29" t="inlineStr">
+      <c r="E16" s="29" t="inlineStr">
         <is>
           <t>ldh [mm]</t>
         </is>
       </c>
-      <c r="F15" s="29" t="inlineStr">
-        <is>
-          <t>Longitud de barra [m]</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="31" t="inlineStr">
-        <is>
-          <t>Viga de carga VC</t>
-        </is>
-      </c>
-      <c r="C16" s="31" t="inlineStr">
-        <is>
-          <t>Nº 5</t>
-        </is>
-      </c>
-      <c r="D16" s="35" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="E16" s="31">
-        <f>F12</f>
-        <v/>
-      </c>
-      <c r="F16" s="34">
-        <f>(D16*1000+2*E16)/1000</f>
-        <v/>
+      <c r="F16" s="29" t="inlineStr">
+        <is>
+          <t>Formula</t>
+        </is>
+      </c>
+      <c r="G16" s="29" t="inlineStr">
+        <is>
+          <t>Longitud [m]</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="31" t="inlineStr">
         <is>
-          <t>Riostra VR</t>
+          <t>Viga superior (apoyos)</t>
         </is>
       </c>
       <c r="C17" s="31" t="inlineStr">
         <is>
-          <t>Nº 5</t>
+          <t>Nº 4</t>
         </is>
       </c>
       <c r="D17" s="35" t="n">
         <v>5.1</v>
       </c>
       <c r="E17" s="31">
-        <f>F12</f>
-        <v/>
-      </c>
-      <c r="F17" s="34">
-        <f>(D17*1000+2*E17)/1000</f>
+        <f>F11</f>
+        <v/>
+      </c>
+      <c r="F17" s="37" t="inlineStr">
+        <is>
+          <t>Ln/4 + ldh</t>
+        </is>
+      </c>
+      <c r="G17" s="34">
+        <f>(D17/4*1000+E17)/1000</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="31" t="inlineStr">
         <is>
-          <t>Vigueta</t>
+          <t>Viga inferior (centro)</t>
         </is>
       </c>
       <c r="C18" s="31" t="inlineStr">
         <is>
-          <t>Nº 4</t>
+          <t>Nº 5</t>
         </is>
       </c>
       <c r="D18" s="35" t="n">
-        <v>4.8</v>
+        <v>5.1</v>
       </c>
       <c r="E18" s="31">
-        <f>F11</f>
-        <v/>
-      </c>
-      <c r="F18" s="34">
+        <f>F12</f>
+        <v/>
+      </c>
+      <c r="F18" s="37" t="inlineStr">
+        <is>
+          <t>Ln + 2 ldh</t>
+        </is>
+      </c>
+      <c r="G18" s="34">
         <f>(D18*1000+2*E18)/1000</f>
         <v/>
       </c>
     </row>
+    <row r="19">
+      <c r="B19" s="31" t="inlineStr">
+        <is>
+          <t>Vigueta superior (apoyos)</t>
+        </is>
+      </c>
+      <c r="C19" s="31" t="inlineStr">
+        <is>
+          <t>Nº 3</t>
+        </is>
+      </c>
+      <c r="D19" s="35" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="E19" s="31">
+        <f>F10</f>
+        <v/>
+      </c>
+      <c r="F19" s="31" t="inlineStr">
+        <is>
+          <t>Ln/4 + ldh</t>
+        </is>
+      </c>
+      <c r="G19" s="34">
+        <f>(D19/4*1000+E19)/1000</f>
+        <v/>
+      </c>
+    </row>
     <row r="20" ht="28" customHeight="1">
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>La longitud incluye un gancho estandar a 90 grados en cada extremo, anclado dentro de las columnas. Para las barras superiores que no se cortan, el baston negativo se extiende Ln/4 mas la longitud de desarrollo desde la cara del apoyo.</t>
-        </is>
+      <c r="B20" s="31" t="inlineStr">
+        <is>
+          <t>Vigueta inferior (centro)</t>
+        </is>
+      </c>
+      <c r="C20" s="31" t="inlineStr">
+        <is>
+          <t>Nº 3</t>
+        </is>
+      </c>
+      <c r="D20" s="35" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="E20" s="31">
+        <f>F10</f>
+        <v/>
+      </c>
+      <c r="F20" s="31" t="inlineStr">
+        <is>
+          <t>Ln + 2 ldh</t>
+        </is>
+      </c>
+      <c r="G20" s="34">
+        <f>(D20*1000+2*E20)/1000</f>
+        <v/>
       </c>
     </row>
     <row r="22">
@@ -6515,10 +6576,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="B28:I28"/>
+    <mergeCell ref="B15:I15"/>
     <mergeCell ref="B6:I6"/>
     <mergeCell ref="B2:I2"/>
-    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="B28:I28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mejorar presentacion del Excel de diseno (portada/indice, colores de pestana, sin cuadricula, impresion) sin cambiar calculos
</commit_message>
<xml_diff>
--- a/Proyectos/Diseno-Estructural/Insumos/Diseno-Estructural-Calculos.xlsx
+++ b/Proyectos/Diseno-Estructural/Insumos/Diseno-Estructural-Calculos.xlsx
@@ -7,13 +7,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Irregularidades" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro Viguetas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro Vigas-Riostras" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diseno Vigas" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diseno Riostras" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diseno Viguetas" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Despiece y Longitudes" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portada" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Irregularidades" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro Viguetas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro Vigas-Riostras" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diseno Vigas" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diseno Riostras" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diseno Viguetas" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Despiece y Longitudes" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,8 +70,59 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <color rgb="00000000"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -100,6 +152,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E5496"/>
       </patternFill>
     </fill>
   </fills>
@@ -184,7 +246,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -278,6 +340,39 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -641,8 +736,226 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="001F3864"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:E19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="38" t="inlineStr">
+        <is>
+          <t>SSS CONSTRUCCIONES Y CONSULTORIAS SAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="39" t="inlineStr">
+        <is>
+          <t>PROYECTO: EDIFICIO RESIDENCIAL SANTA MARTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="40" t="inlineStr">
+        <is>
+          <t>MEMORIA DE CALCULO ESTRUCTURAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="41" t="inlineStr">
+        <is>
+          <t>Diseno de viguetas, vigas y riostras - NSR-10 / ACI 318</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="42" t="inlineStr">
+        <is>
+          <t>CONTENIDO DEL LIBRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="43" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="C9" s="44" t="inlineStr">
+        <is>
+          <t>Hoja</t>
+        </is>
+      </c>
+      <c r="D9" s="44" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C10" s="46" t="inlineStr">
+        <is>
+          <t>Irregularidades</t>
+        </is>
+      </c>
+      <c r="D10" s="47" t="inlineStr">
+        <is>
+          <t>Sistema, R0, Omega0, irregularidades (R = 5.0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="45" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C11" s="46" t="inlineStr">
+        <is>
+          <t>Cuadro Viguetas</t>
+        </is>
+      </c>
+      <c r="D11" s="47" t="inlineStr">
+        <is>
+          <t>Diseno por tipo de luz (entrepiso y cubierta)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="45" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C12" s="46" t="inlineStr">
+        <is>
+          <t>Cuadro Vigas-Riostras</t>
+        </is>
+      </c>
+      <c r="D12" s="47" t="inlineStr">
+        <is>
+          <t>Diseno por tipos de solicitacion</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="45" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C13" s="46" t="inlineStr">
+        <is>
+          <t>Diseno Vigas</t>
+        </is>
+      </c>
+      <c r="D13" s="47" t="inlineStr">
+        <is>
+          <t>Calculo detallado viga critica VC-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="45" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C14" s="46" t="inlineStr">
+        <is>
+          <t>Diseno Riostras</t>
+        </is>
+      </c>
+      <c r="D14" s="47" t="inlineStr">
+        <is>
+          <t>Calculo detallado riostra critica VR-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="45" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C15" s="46" t="inlineStr">
+        <is>
+          <t>Diseno Viguetas</t>
+        </is>
+      </c>
+      <c r="D15" s="47" t="inlineStr">
+        <is>
+          <t>Calculo detallado vigueta critica</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="45" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C16" s="46" t="inlineStr">
+        <is>
+          <t>Despiece y Longitudes</t>
+        </is>
+      </c>
+      <c r="D16" s="47" t="inlineStr">
+        <is>
+          <t>Ganchos, longitud de barras y estribos</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="48" t="inlineStr">
+        <is>
+          <t>Materiales: f'c = 28 MPa, fy = 420 MPa.  Sistema: porticos de concreto DMO.  Localizacion: Santa Marta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="48" t="inlineStr">
+        <is>
+          <t>Responsables: Sergio Bolivar, Santiago Ospina, Cristian Bautista.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="B18:E18"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B19:E19"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00C00000"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B2:J72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1784,15 +2097,26 @@
     <mergeCell ref="B5:J8"/>
     <mergeCell ref="B2:J2"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.7" bottom="0.7" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;"Aptos Narrow"&amp;8 EDIFICIO RESIDENCIAL SANTA MARTA&amp;R&amp;"Aptos Narrow"&amp;8 SSS Construcciones y Consultorias SAS</oddHeader>
+    <oddFooter>&amp;C&amp;8 Pagina &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00548235"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B2:N29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -2602,15 +2926,26 @@
     <mergeCell ref="B10:N10"/>
     <mergeCell ref="B27:N29"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.7" bottom="0.7" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;"Aptos Narrow"&amp;8 EDIFICIO RESIDENCIAL SANTA MARTA&amp;R&amp;"Aptos Narrow"&amp;8 SSS Construcciones y Consultorias SAS</oddHeader>
+    <oddFooter>&amp;C&amp;8 Pagina &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00548235"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B2:O25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -3301,15 +3636,26 @@
     <mergeCell ref="B7:O7"/>
     <mergeCell ref="B23:O25"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.7" bottom="0.7" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;"Aptos Narrow"&amp;8 EDIFICIO RESIDENCIAL SANTA MARTA&amp;R&amp;"Aptos Narrow"&amp;8 SSS Construcciones y Consultorias SAS</oddHeader>
+    <oddFooter>&amp;C&amp;8 Pagina &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="002E5496"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B2:J80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -4328,15 +4674,26 @@
     <mergeCell ref="B79:J80"/>
     <mergeCell ref="B2:J2"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.7" bottom="0.7" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;"Aptos Narrow"&amp;8 EDIFICIO RESIDENCIAL SANTA MARTA&amp;R&amp;"Aptos Narrow"&amp;8 SSS Construcciones y Consultorias SAS</oddHeader>
+    <oddFooter>&amp;C&amp;8 Pagina &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="002E5496"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B2:J80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -5355,15 +5712,26 @@
     <mergeCell ref="B79:J80"/>
     <mergeCell ref="B2:J2"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.7" bottom="0.7" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;"Aptos Narrow"&amp;8 EDIFICIO RESIDENCIAL SANTA MARTA&amp;R&amp;"Aptos Narrow"&amp;8 SSS Construcciones y Consultorias SAS</oddHeader>
+    <oddFooter>&amp;C&amp;8 Pagina &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="002E5496"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B2:J56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -6035,15 +6403,26 @@
     <mergeCell ref="B55:J56"/>
     <mergeCell ref="B2:J2"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.7" bottom="0.7" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;"Aptos Narrow"&amp;8 EDIFICIO RESIDENCIAL SANTA MARTA&amp;R&amp;"Aptos Narrow"&amp;8 SSS Construcciones y Consultorias SAS</oddHeader>
+    <oddFooter>&amp;C&amp;8 Pagina &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00BF8F00"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B2:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -6576,11 +6955,21 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="B15:I15"/>
+    <mergeCell ref="B28:I28"/>
     <mergeCell ref="B6:I6"/>
     <mergeCell ref="B2:I2"/>
-    <mergeCell ref="B28:I28"/>
+    <mergeCell ref="B15:I15"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.7" bottom="0.7" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;"Aptos Narrow"&amp;8 EDIFICIO RESIDENCIAL SANTA MARTA&amp;R&amp;"Aptos Narrow"&amp;8 SSS Construcciones y Consultorias SAS</oddHeader>
+    <oddFooter>&amp;C&amp;8 Pagina &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Alinear ejemplos detallados (Diseno Vigas/Riostras y memoria) con el cuadro: VC-3 M+=79 (4N5), VR-4 M-=243/M+=134, eliminando inconsistencia de momentos
</commit_message>
<xml_diff>
--- a/Proyectos/Diseno-Estructural/Insumos/Diseno-Estructural-Calculos.xlsx
+++ b/Proyectos/Diseno-Estructural/Insumos/Diseno-Estructural-Calculos.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portada" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Irregularidades" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro Viguetas" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro Vigas-Riostras" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diseno Vigas" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diseno Riostras" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diseno Viguetas" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Despiece y Longitudes" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Portada" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Irregularidades" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Cuadro Viguetas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cuadro Vigas-Riostras" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Diseno Vigas" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Diseno Riostras" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Diseno Viguetas" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Despiece y Longitudes" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3891,7 +3891,7 @@
         </is>
       </c>
       <c r="C19" s="5" t="n">
-        <v>101</v>
+        <v>79</v>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
@@ -4914,7 +4914,7 @@
         </is>
       </c>
       <c r="C18" s="5" t="n">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
@@ -4929,7 +4929,7 @@
         </is>
       </c>
       <c r="C19" s="5" t="n">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Agregar diseno paso a paso de viguetas de entrepiso y de cubierta (viga T, gravedad)
</commit_message>
<xml_diff>
--- a/Proyectos/Diseno-Estructural/Insumos/Diseno-Estructural-Calculos.xlsx
+++ b/Proyectos/Diseno-Estructural/Insumos/Diseno-Estructural-Calculos.xlsx
@@ -18,8 +18,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diseno VR-2" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diseno VR-3" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diseno VR-4" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diseno Viguetas" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Despiece y Longitudes" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diseno Vigueta Entrepiso" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diseno Vigueta Cubierta" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Despiece y Longitudes" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -745,7 +746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E21"/>
+  <dimension ref="B2:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -926,15 +927,12 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="B18" s="48" t="n"/>
     </row>
     <row r="19">
       <c r="B19" s="48" t="n"/>
     </row>
-    <row r="20"/>
-    <row r="21"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="B18:E18"/>
@@ -2965,11 +2963,11 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="002E5496"/>
+    <tabColor rgb="00548235"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:J56"/>
+  <dimension ref="B2:J52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -2981,13 +2979,13 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="46" customWidth="1" min="10" max="10"/>
+    <col width="44" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>DISENO DE VIGUETAS (losa aligerada en una direccion) - viga T, gravedad</t>
+          <t>DISENO VIGUETA DE ENTREPISO  (losa aligerada, viga T)</t>
         </is>
       </c>
     </row>
@@ -2999,7 +2997,7 @@
       </c>
       <c r="J4" s="7" t="inlineStr">
         <is>
-          <t>Celdas azules = entrada</t>
+          <t>Azul = entrada</t>
         </is>
       </c>
     </row>
@@ -3145,7 +3143,7 @@
         </is>
       </c>
       <c r="C14" s="5" t="n">
-        <v>4.75</v>
+        <v>4.8</v>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
@@ -3188,7 +3186,7 @@
     <row r="18">
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>2. CARGAS Y SOLICITACIONES (gravedad)</t>
+          <t>2. CARGAS Y SOLICITACIONES (gravedad - vigueta continua)</t>
         </is>
       </c>
     </row>
@@ -3241,7 +3239,7 @@
     <row r="22">
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Mu (-) = wu Ln2/10</t>
+          <t>Mu (-) = wu Ln2/10 (apoyo)</t>
         </is>
       </c>
       <c r="C22" s="14">
@@ -3257,7 +3255,7 @@
     <row r="23">
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Mu (+) = wu Ln2/14</t>
+          <t>Mu (+) = wu Ln2/14 (centro)</t>
         </is>
       </c>
       <c r="C23" s="14">
@@ -3588,7 +3586,7 @@
     <row r="50">
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>6. DEFLEXION (C.9.5)</t>
+          <t>6. DEFLEXION</t>
         </is>
       </c>
     </row>
@@ -3619,32 +3617,15 @@
         <v/>
       </c>
     </row>
-    <row r="54">
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>7. DESPIECE</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="40" customHeight="1">
-      <c r="B55" s="7" t="inlineStr">
-        <is>
-          <t>Refuerzo inferior As(+) corrido en el nervio; superior As(-) sobre apoyos (bastones Ln/4 + ld). Loseta con malla de retraccion (As=0.0018 b hf). Sin estribos si Vu &lt;= phi 1.1 Vc.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56"/>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B55:J56"/>
+  <mergeCells count="1">
     <mergeCell ref="B2:J2"/>
   </mergeCells>
-  <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.4" right="0.4" top="0.7" bottom="0.7" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;L&amp;"Aptos Narrow"&amp;8 EDIFICIO RESIDENCIAL SANTA MARTA&amp;R&amp;"Aptos Narrow"&amp;8 SSS Construcciones y Consultorias SAS</oddHeader>
-    <oddFooter>&amp;C&amp;8 Pagina &amp;P de &amp;N</oddFooter>
+    <oddHeader>&amp;LEDIFICIO RESIDENCIAL SANTA MARTA&amp;RSSS Construcciones SAS</oddHeader>
+    <oddFooter>&amp;CPagina &amp;P de &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -3654,6 +3635,680 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00548235"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B2:J52"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="44" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>DISENO VIGUETA DE CUBIERTA - terraza social L=5 (viga T)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>1. DATOS Y GEOMETRIA</t>
+        </is>
+      </c>
+      <c r="J4" s="7" t="inlineStr">
+        <is>
+          <t>Azul = entrada</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>f'c</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>fy</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>420</v>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>bw (nervio)</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>h (total)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>hf (loseta)</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>separacion sv</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>recubrimiento r</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Diam barra long.</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>mm #4</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Area barra</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>129</v>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>mm2 #4</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Luz libre Ln</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>d = h - r - bl/2</t>
+        </is>
+      </c>
+      <c r="C15" s="14">
+        <f>C8*1000-C11*1000-C12/2</f>
+        <v/>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>bf = min(Ln/4 ; bw+16hf ; sv)</t>
+        </is>
+      </c>
+      <c r="C16" s="14">
+        <f>MIN(C14*1000/4,C7*1000+16*C9*1000,C10*1000)</f>
+        <v/>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>2. CARGAS Y SOLICITACIONES (gravedad - vigueta continua)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Carga muerta wD</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>4.376</v>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>kN/m2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Carga viva wL</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>kN/m2</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>wu = (1.2D+1.6L) sv</t>
+        </is>
+      </c>
+      <c r="C21" s="14">
+        <f>(1.2*C19+1.6*C20)*C10</f>
+        <v/>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>kN/m</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Mu (-) = wu Ln2/10 (apoyo)</t>
+        </is>
+      </c>
+      <c r="C22" s="14">
+        <f>C21*C14^2/10</f>
+        <v/>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>kN.m</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Mu (+) = wu Ln2/14 (centro)</t>
+        </is>
+      </c>
+      <c r="C23" s="14">
+        <f>C21*C14^2/14</f>
+        <v/>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>kN.m</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Vu = 1.15 wu Ln/2</t>
+        </is>
+      </c>
+      <c r="C24" s="14">
+        <f>1.15*C21*C14/2</f>
+        <v/>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>kN</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>3. FLEXION POSITIVA - viga T (loseta a compresion, ancho bf)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Rn = Mu+/(phi bf d2)</t>
+        </is>
+      </c>
+      <c r="C27" s="9">
+        <f>C23*1000000/(0.9*C16*C15^2)</f>
+        <v/>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>rho</t>
+        </is>
+      </c>
+      <c r="C28" s="9">
+        <f>(0.85*C5/C6)*(1-SQRT(1-2*C27/(0.85*C5)))</f>
+        <v/>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>As+</t>
+        </is>
+      </c>
+      <c r="C29" s="9">
+        <f>C28*C16*C15</f>
+        <v/>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>a = As fy/(0.85 f'c bf)</t>
+        </is>
+      </c>
+      <c r="C30" s="9">
+        <f>C29*C6/(0.85*C5*C16)</f>
+        <v/>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>a &lt;= hf? (T verdadera)</t>
+        </is>
+      </c>
+      <c r="C31" s="9">
+        <f>IF(C30&lt;=C9*1000,"Si (bloque en loseta)","revisar T real")</f>
+        <v/>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>As minimo</t>
+        </is>
+      </c>
+      <c r="C32" s="9">
+        <f>MAX(0.25*SQRT(C5)/C6,1.4/C6)*C7*1000*C15</f>
+        <v/>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>As+ de diseno</t>
+        </is>
+      </c>
+      <c r="C33" s="15">
+        <f>MAX(C29,C32)</f>
+        <v/>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>N barras (#4)</t>
+        </is>
+      </c>
+      <c r="C34" s="14">
+        <f>ROUNDUP(C33/C13,0)</f>
+        <v/>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>u</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>VERIFICACION flexion (+)</t>
+        </is>
+      </c>
+      <c r="C35" s="11">
+        <f>IF(AND(C33&gt;=C32,C30&lt;=C9*1000),"CUMPLE","REVISAR")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>4. FLEXION NEGATIVA - rectangular (nervio bw)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Rn = Mu-/(phi bw d2)</t>
+        </is>
+      </c>
+      <c r="C38" s="9">
+        <f>C22*1000000/(0.9*C7*1000*C15^2)</f>
+        <v/>
+      </c>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>rho</t>
+        </is>
+      </c>
+      <c r="C39" s="9">
+        <f>(0.85*C5/C6)*(1-SQRT(1-2*C38/(0.85*C5)))</f>
+        <v/>
+      </c>
+      <c r="D39" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>As-</t>
+        </is>
+      </c>
+      <c r="C40" s="9">
+        <f>C39*C7*1000*C15</f>
+        <v/>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>As- de diseno (&gt;= min)</t>
+        </is>
+      </c>
+      <c r="C41" s="15">
+        <f>MAX(C40,C32)</f>
+        <v/>
+      </c>
+      <c r="D41" s="9" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>N barras (#4)</t>
+        </is>
+      </c>
+      <c r="C42" s="14">
+        <f>ROUNDUP(C41/C13,0)</f>
+        <v/>
+      </c>
+      <c r="D42" s="9" t="inlineStr">
+        <is>
+          <t>u</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>VERIFICACION flexion (-)</t>
+        </is>
+      </c>
+      <c r="C43" s="11">
+        <f>IF(C41&gt;=C32,"CUMPLE","REVISAR")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>5. CORTANTE (vigueta: Vc +10% - C.8.13.8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Vc = 0.17 raiz(f'c) bw d</t>
+        </is>
+      </c>
+      <c r="C46" s="9">
+        <f>0.17*SQRT(C5)*C7*1000*C15/1000</f>
+        <v/>
+      </c>
+      <c r="D46" s="9" t="inlineStr">
+        <is>
+          <t>kN</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>phi 1.1 Vc</t>
+        </is>
+      </c>
+      <c r="C47" s="9">
+        <f>0.75*1.1*C46</f>
+        <v/>
+      </c>
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>kN</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Vu &lt;= phi 1.1 Vc?</t>
+        </is>
+      </c>
+      <c r="C48" s="11">
+        <f>IF(C24&lt;=C47,"Si - sin estribos","Requiere estribos")</f>
+        <v/>
+      </c>
+      <c r="D48" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>6. DEFLEXION</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>h min = Ln/18.5</t>
+        </is>
+      </c>
+      <c r="C51" s="9">
+        <f>C14/18.5</f>
+        <v/>
+      </c>
+      <c r="D51" s="9" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>VERIFICACION</t>
+        </is>
+      </c>
+      <c r="C52" s="11">
+        <f>IF(C8&gt;=C51,"CUMPLE","REVISAR")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:J2"/>
+  </mergeCells>
+  <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;LEDIFICIO RESIDENCIAL SANTA MARTA&amp;RSSS Construcciones SAS</oddHeader>
+    <oddFooter>&amp;CPagina &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00BF8F00"/>

</xml_diff>